<commit_message>
Added source of contactID and organizationID to notes slot ("sample collected by" "sequence submitted by", "sequenced by", and "isolated by")
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B93460-2AAF-184D-90E5-3DC96730B86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2059E499-1196-2945-ABF6-C0E11981D210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="40720" windowHeight="20600" firstSheet="8" activeTab="10" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="40720" windowHeight="20600" firstSheet="7" activeTab="14" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="accessions_maps" sheetId="12" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9227" uniqueCount="2093">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9237" uniqueCount="2093">
   <si>
     <t>Complete</t>
   </si>
@@ -6757,7 +6757,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -6911,19 +6911,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -30250,10 +30237,10 @@
       <c r="G85" t="s">
         <v>958</v>
       </c>
-      <c r="K85" s="78" t="s">
+      <c r="K85" t="s">
         <v>1115</v>
       </c>
-      <c r="L85" s="78" t="s">
+      <c r="L85" t="s">
         <v>1115</v>
       </c>
       <c r="O85" t="s">
@@ -30307,10 +30294,10 @@
       <c r="G86" t="s">
         <v>958</v>
       </c>
-      <c r="K86" s="78" t="s">
+      <c r="K86" t="s">
         <v>1115</v>
       </c>
-      <c r="L86" s="78" t="s">
+      <c r="L86" t="s">
         <v>1115</v>
       </c>
       <c r="O86" t="s">
@@ -30364,10 +30351,10 @@
       <c r="G87" t="s">
         <v>958</v>
       </c>
-      <c r="K87" s="78" t="s">
+      <c r="K87" t="s">
         <v>1115</v>
       </c>
-      <c r="L87" s="78" t="s">
+      <c r="L87" t="s">
         <v>1115</v>
       </c>
       <c r="O87" t="s">
@@ -32797,17 +32784,18 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0435B3-2676-7B49-A30C-B02B45DA7889}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="28.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.1640625" customWidth="1"/>
+    <col min="12" max="12" width="29.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
         <v>1721</v>
       </c>
@@ -32838,11 +32826,14 @@
       <c r="J1" s="18" t="s">
         <v>1806</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="18" t="s">
+        <v>1791</v>
+      </c>
+      <c r="L1" s="25" t="s">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B2" t="b">
         <v>1</v>
       </c>
@@ -32865,10 +32856,17 @@
       <c r="K2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B3" t="b">
         <v>1</v>
+      </c>
+      <c r="C3" t="str">
+        <f>IF(E3&lt;&gt;"",VLOOKUP(E3,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v>Sequence information</v>
       </c>
       <c r="D3" t="s">
         <v>1809</v>
@@ -32885,10 +32883,17 @@
       <c r="K3" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B4" t="b">
         <v>1</v>
+      </c>
+      <c r="C4" t="str">
+        <f>IF(E4&lt;&gt;"",VLOOKUP(E4,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v>Sequence information</v>
       </c>
       <c r="D4" t="s">
         <v>1809</v>
@@ -32905,10 +32910,17 @@
       <c r="K4" t="s">
         <v>1115</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" t="s">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B5" t="b">
         <v>1</v>
+      </c>
+      <c r="C5" t="str">
+        <f>IF(E5&lt;&gt;"",VLOOKUP(E5,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v>Strain and isolation information</v>
       </c>
       <c r="D5" t="s">
         <v>1809</v>
@@ -32923,6 +32935,9 @@
         <v>1476</v>
       </c>
       <c r="K5" t="s">
+        <v>1107</v>
+      </c>
+      <c r="L5" t="s">
         <v>1107</v>
       </c>
     </row>
@@ -33186,446 +33201,444 @@
   <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="25.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.33203125" style="82" customWidth="1"/>
-    <col min="2" max="6" width="25.33203125" style="82"/>
-    <col min="7" max="7" width="44" style="82" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="25.33203125" style="82"/>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="7" max="7" width="44" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="84" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+    <row r="1" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="24" t="s">
         <v>1411</v>
       </c>
-      <c r="B1" s="83" t="s">
+      <c r="B1" s="24" t="s">
         <v>1721</v>
       </c>
-      <c r="C1" s="83" t="s">
+      <c r="C1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="83" t="s">
+      <c r="D1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="83" t="s">
+      <c r="E1" s="24" t="s">
         <v>1821</v>
       </c>
-      <c r="F1" s="83" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="83" t="s">
+      <c r="F1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="83" t="s">
+      <c r="H1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="83" t="s">
+      <c r="I1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="83" t="s">
+      <c r="J1" s="24" t="s">
         <v>1742</v>
       </c>
-      <c r="K1" s="83" t="s">
+      <c r="K1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="83" t="s">
+      <c r="L1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="83" t="s">
+      <c r="M1" s="24" t="s">
         <v>1728</v>
       </c>
-      <c r="N1" s="83" t="s">
+      <c r="N1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="83" t="s">
+      <c r="O1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="83" t="s">
+      <c r="P1" s="24" t="s">
         <v>1719</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="81">
+      <c r="A2" s="23">
         <v>3</v>
       </c>
-      <c r="B2" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C2" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" s="81" t="s">
+      <c r="B2" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>1121</v>
       </c>
-      <c r="E2" s="82" t="str">
+      <c r="E2" t="str">
         <f>IF(G2&lt;&gt;"",VLOOKUP(G2,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>AMR detection information</v>
       </c>
-      <c r="F2" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G2" s="81" t="s">
+      <c r="F2" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G2" s="23" t="s">
         <v>1123</v>
       </c>
-      <c r="H2" s="81" t="s">
+      <c r="H2" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I2" s="81" t="s">
+      <c r="I2" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81" t="s">
+      <c r="J2" s="23"/>
+      <c r="K2" s="23" t="s">
         <v>1564</v>
       </c>
-      <c r="L2" s="81" t="s">
+      <c r="L2" s="23" t="s">
         <v>1693</v>
       </c>
-      <c r="M2" s="81"/>
-      <c r="N2" s="81"/>
-      <c r="O2" s="81" t="s">
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23" t="s">
         <v>1565</v>
       </c>
-      <c r="P2" s="81" t="s">
+      <c r="P2" s="23" t="s">
         <v>1720</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="81">
+      <c r="A3" s="23">
         <v>10</v>
       </c>
-      <c r="B3" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" s="81" t="s">
+      <c r="B3" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="82" t="str">
+      <c r="E3" t="str">
         <f>IF(G3&lt;&gt;"",VLOOKUP(G3,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F3" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G3" s="81" t="s">
+      <c r="F3" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G3" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="81" t="s">
+      <c r="H3" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I3" s="81" t="s">
+      <c r="I3" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81" t="s">
+      <c r="J3" s="23"/>
+      <c r="K3" s="23" t="s">
         <v>1564</v>
       </c>
-      <c r="L3" s="81" t="s">
+      <c r="L3" s="23" t="s">
         <v>1697</v>
       </c>
-      <c r="M3" s="81"/>
-      <c r="N3" s="81"/>
-      <c r="O3" s="81" t="s">
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23" t="s">
         <v>1573</v>
       </c>
-      <c r="P3" s="81"/>
+      <c r="P3" s="23"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A4" s="81">
+      <c r="A4" s="23">
         <v>46</v>
       </c>
-      <c r="B4" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D4" s="81" t="s">
+      <c r="B4" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="82" t="str">
+      <c r="E4" t="str">
         <f>IF(G4&lt;&gt;"",VLOOKUP(G4,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F4" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G4" s="81" t="s">
+      <c r="F4" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G4" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="H4" s="81" t="s">
+      <c r="H4" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I4" s="81" t="s">
+      <c r="I4" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81" t="s">
+      <c r="J4" s="23"/>
+      <c r="K4" s="23" t="s">
         <v>1564</v>
       </c>
-      <c r="L4" s="81" t="s">
+      <c r="L4" s="23" t="s">
         <v>1679</v>
       </c>
-      <c r="M4" s="81"/>
-      <c r="N4" s="81"/>
-      <c r="O4" s="81" t="s">
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23" t="s">
         <v>1580</v>
       </c>
-      <c r="P4" s="81"/>
+      <c r="P4" s="23"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A5" s="81">
+      <c r="A5" s="23">
         <v>227</v>
       </c>
-      <c r="B5" s="81"/>
-      <c r="C5" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="81" t="s">
+      <c r="B5" s="23"/>
+      <c r="C5" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>1127</v>
       </c>
-      <c r="E5" s="82" t="str">
+      <c r="E5" t="str">
         <f>IF(G5&lt;&gt;"",VLOOKUP(G5,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Lineage/clade information</v>
       </c>
-      <c r="F5" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G5" s="81" t="s">
+      <c r="F5" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G5" s="23" t="s">
         <v>1130</v>
       </c>
-      <c r="H5" s="81" t="s">
+      <c r="H5" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I5" s="81" t="s">
+      <c r="I5" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J5" s="81"/>
-      <c r="K5" s="81" t="s">
+      <c r="J5" s="23"/>
+      <c r="K5" s="23" t="s">
         <v>1564</v>
       </c>
-      <c r="L5" s="81" t="s">
+      <c r="L5" s="23" t="s">
         <v>1680</v>
       </c>
-      <c r="M5" s="81"/>
-      <c r="N5" s="81"/>
-      <c r="O5" s="81" t="s">
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23" t="s">
         <v>1582</v>
       </c>
-      <c r="P5" s="81" t="s">
+      <c r="P5" s="23" t="s">
         <v>1729</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A6" s="81">
+      <c r="A6" s="23">
         <v>330</v>
       </c>
-      <c r="B6" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="81"/>
-      <c r="D6" s="81" t="s">
+      <c r="B6" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E6" s="82" t="e">
+      <c r="E6" t="e">
         <f>IF(G6&lt;&gt;"",VLOOKUP(G6,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="F6" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G6" s="81" t="s">
+      <c r="F6" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G6" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="H6" s="81" t="s">
+      <c r="H6" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I6" s="81" t="s">
+      <c r="I6" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J6" s="81"/>
-      <c r="K6" s="81" t="s">
+      <c r="J6" s="23"/>
+      <c r="K6" s="23" t="s">
         <v>1486</v>
       </c>
-      <c r="L6" s="81" t="s">
+      <c r="L6" s="23" t="s">
         <v>1592</v>
       </c>
-      <c r="M6" s="81"/>
-      <c r="N6" s="81"/>
-      <c r="O6" s="81" t="s">
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23" t="s">
         <v>1591</v>
       </c>
-      <c r="P6" s="81"/>
+      <c r="P6" s="23"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A7" s="81">
+      <c r="A7" s="23">
         <v>331</v>
       </c>
-      <c r="B7" s="81"/>
-      <c r="C7" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="81" t="s">
+      <c r="B7" s="23"/>
+      <c r="C7" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="82" t="str">
+      <c r="E7" t="str">
         <f>IF(G7&lt;&gt;"",VLOOKUP(G7,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="F7" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G7" s="81" t="s">
+      <c r="F7" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G7" s="23" t="s">
         <v>1100</v>
       </c>
-      <c r="H7" s="81" t="s">
+      <c r="H7" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I7" s="81" t="s">
+      <c r="I7" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J7" s="81"/>
-      <c r="K7" s="81" t="s">
+      <c r="J7" s="23"/>
+      <c r="K7" s="23" t="s">
         <v>1486</v>
       </c>
-      <c r="L7" s="81" t="s">
+      <c r="L7" s="23" t="s">
         <v>1595</v>
       </c>
-      <c r="M7" s="81"/>
-      <c r="N7" s="81"/>
-      <c r="O7" s="81" t="s">
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23" t="s">
         <v>1596</v>
       </c>
-      <c r="P7" s="81" t="s">
+      <c r="P7" s="23" t="s">
         <v>1732</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="81">
+      <c r="A8" s="23">
         <v>659</v>
       </c>
-      <c r="B8" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="81" t="s">
+      <c r="B8" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="82" t="str">
+      <c r="E8" t="str">
         <f>IF(G8&lt;&gt;"",VLOOKUP(G8,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="F8" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G8" s="85" t="s">
+      <c r="F8" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G8" s="77" t="s">
         <v>1839</v>
       </c>
-      <c r="H8" s="86" t="s">
+      <c r="H8" s="40" t="s">
         <v>442</v>
       </c>
-      <c r="I8" s="81" t="s">
+      <c r="I8" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J8" s="81"/>
-      <c r="K8" s="81" t="s">
+      <c r="J8" s="23"/>
+      <c r="K8" s="23" t="s">
         <v>1486</v>
       </c>
-      <c r="L8" s="81" t="s">
+      <c r="L8" s="23" t="s">
         <v>1308</v>
       </c>
-      <c r="M8" s="81"/>
-      <c r="N8" s="81"/>
-      <c r="O8" s="81" t="s">
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23" t="s">
         <v>1604</v>
       </c>
-      <c r="P8" s="81"/>
+      <c r="P8" s="23"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A9" s="81">
+      <c r="A9" s="23">
         <v>717</v>
       </c>
-      <c r="B9" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="81" t="s">
+      <c r="B9" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="82" t="str">
+      <c r="E9" t="str">
         <f>IF(G9&lt;&gt;"",VLOOKUP(G9,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="F9" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G9" s="81" t="s">
+      <c r="F9" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G9" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="H9" s="81" t="s">
+      <c r="H9" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I9" s="81" t="s">
+      <c r="I9" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J9" s="81"/>
-      <c r="K9" s="81" t="s">
+      <c r="J9" s="23"/>
+      <c r="K9" s="23" t="s">
         <v>1486</v>
       </c>
-      <c r="L9" s="81" t="s">
+      <c r="L9" s="23" t="s">
         <v>1485</v>
       </c>
-      <c r="M9" s="81"/>
-      <c r="N9" s="81"/>
-      <c r="O9" s="81" t="s">
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23" t="s">
         <v>1484</v>
       </c>
-      <c r="P9" s="81"/>
+      <c r="P9" s="23"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A10" s="81">
+      <c r="A10" s="23">
         <v>846</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" s="81" t="s">
+      <c r="B10" s="23"/>
+      <c r="C10" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>1118</v>
       </c>
-      <c r="E10" s="82" t="str">
+      <c r="E10" t="str">
         <f>IF(G10&lt;&gt;"",VLOOKUP(G10,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Taxonomic identification information</v>
       </c>
-      <c r="F10" s="81" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G10" s="81" t="s">
+      <c r="F10" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="H10" s="81" t="s">
+      <c r="H10" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I10" s="81" t="s">
+      <c r="I10" s="23" t="s">
         <v>1237</v>
       </c>
-      <c r="J10" s="81"/>
-      <c r="K10" s="81" t="s">
+      <c r="J10" s="23"/>
+      <c r="K10" s="23" t="s">
         <v>1564</v>
       </c>
-      <c r="L10" s="81" t="s">
+      <c r="L10" s="23" t="s">
         <v>1650</v>
       </c>
-      <c r="M10" s="81"/>
-      <c r="N10" s="81"/>
-      <c r="O10" s="81" t="s">
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23" t="s">
         <v>1649</v>
       </c>
-      <c r="P10" s="81"/>
+      <c r="P10" s="23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -49142,554 +49155,551 @@
   <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="80" customWidth="1"/>
-    <col min="2" max="2" width="15" style="80" customWidth="1"/>
-    <col min="3" max="3" width="10.5" style="80" customWidth="1"/>
-    <col min="4" max="5" width="26.1640625" style="80" customWidth="1"/>
-    <col min="6" max="6" width="13" style="80" customWidth="1"/>
-    <col min="7" max="7" width="25" style="80" customWidth="1"/>
-    <col min="8" max="8" width="34.5" style="80" customWidth="1"/>
-    <col min="9" max="9" width="13" style="80" customWidth="1"/>
-    <col min="10" max="10" width="6.6640625" style="80" customWidth="1"/>
-    <col min="11" max="11" width="10.5" style="80" customWidth="1"/>
-    <col min="12" max="13" width="20.83203125" style="80" customWidth="1"/>
-    <col min="14" max="14" width="7.5" style="80" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" style="80" customWidth="1"/>
-    <col min="16" max="16" width="62.33203125" style="80" customWidth="1"/>
-    <col min="17" max="17" width="13" style="80" customWidth="1"/>
-    <col min="18" max="16384" width="10.83203125" style="80"/>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="10.5" customWidth="1"/>
+    <col min="4" max="5" width="26.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="25" customWidth="1"/>
+    <col min="8" max="8" width="34.5" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="6.6640625" customWidth="1"/>
+    <col min="11" max="11" width="10.5" customWidth="1"/>
+    <col min="12" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="7.5" customWidth="1"/>
+    <col min="15" max="15" width="12.6640625" customWidth="1"/>
+    <col min="16" max="16" width="62.33203125" customWidth="1"/>
+    <col min="17" max="17" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="84" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="83" t="s">
+    <row r="1" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="24" t="s">
         <v>1411</v>
       </c>
-      <c r="B1" s="83" t="s">
+      <c r="B1" s="24" t="s">
         <v>1721</v>
       </c>
-      <c r="C1" s="83" t="s">
+      <c r="C1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="83" t="s">
+      <c r="D1" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="83" t="s">
+      <c r="E1" s="24" t="s">
         <v>1821</v>
       </c>
-      <c r="F1" s="83" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="83" t="s">
+      <c r="F1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="83" t="s">
+      <c r="H1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="83" t="s">
+      <c r="I1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="83" t="s">
+      <c r="J1" s="24" t="s">
         <v>1742</v>
       </c>
-      <c r="K1" s="83" t="s">
+      <c r="K1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="83" t="s">
+      <c r="L1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="83" t="s">
+      <c r="M1" s="24" t="s">
         <v>1780</v>
       </c>
-      <c r="N1" s="83" t="s">
+      <c r="N1" s="24" t="s">
         <v>1728</v>
       </c>
-      <c r="O1" s="83" t="s">
+      <c r="O1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="83" t="s">
+      <c r="P1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="Q1" s="83" t="s">
+      <c r="Q1" s="24" t="s">
         <v>1719</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="79">
+      <c r="A2" s="23">
         <v>25</v>
       </c>
-      <c r="B2" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C2" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D2" s="79" t="s">
+      <c r="B2" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="80" t="str">
+      <c r="E2" t="str">
         <f>IF(G2&lt;&gt;"",VLOOKUP(G2,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F2" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G2" s="79" t="s">
+      <c r="F2" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G2" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="H2" s="79" t="s">
+      <c r="H2" s="23" t="s">
         <v>442</v>
       </c>
-      <c r="I2" s="79" t="s">
+      <c r="I2" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79" t="s">
+      <c r="J2" s="23"/>
+      <c r="K2" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="79" t="s">
+      <c r="L2" s="23" t="s">
         <v>1274</v>
       </c>
-      <c r="M2" s="79"/>
-      <c r="N2" s="79"/>
-      <c r="O2" s="79"/>
-      <c r="P2" s="79" t="s">
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q2" s="79" t="s">
+      <c r="Q2" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A3" s="79">
+      <c r="A3" s="23">
         <v>32</v>
       </c>
-      <c r="B3" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C3" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D3" s="79" t="s">
+      <c r="B3" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="80" t="str">
+      <c r="E3" t="str">
         <f>IF(G3&lt;&gt;"",VLOOKUP(G3,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F3" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G3" s="79" t="s">
+      <c r="F3" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G3" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H3" s="79" t="s">
+      <c r="H3" s="23" t="s">
         <v>2075</v>
       </c>
-      <c r="I3" s="79" t="s">
+      <c r="I3" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J3" s="79"/>
-      <c r="K3" s="79" t="s">
+      <c r="J3" s="23"/>
+      <c r="K3" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L3" s="79" t="s">
+      <c r="L3" s="23" t="s">
         <v>1262</v>
       </c>
-      <c r="M3" s="79"/>
-      <c r="N3" s="79"/>
-      <c r="O3" s="79"/>
-      <c r="P3" s="79" t="s">
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q3" s="79" t="s">
+      <c r="Q3" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A4" s="79">
+      <c r="A4" s="23">
         <v>33</v>
       </c>
-      <c r="B4" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C4" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D4" s="79" t="s">
+      <c r="B4" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="80" t="str">
+      <c r="E4" t="str">
         <f>IF(G4&lt;&gt;"",VLOOKUP(G4,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F4" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G4" s="79" t="s">
+      <c r="F4" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G4" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H4" s="79" t="s">
+      <c r="H4" s="23" t="s">
         <v>2076</v>
       </c>
-      <c r="I4" s="79" t="s">
+      <c r="I4" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79" t="s">
+      <c r="J4" s="23"/>
+      <c r="K4" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L4" s="79" t="s">
+      <c r="L4" s="23" t="s">
         <v>1263</v>
       </c>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="79"/>
-      <c r="P4" s="79" t="s">
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q4" s="79" t="s">
+      <c r="Q4" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A5" s="79">
+      <c r="A5" s="23">
         <v>34</v>
       </c>
-      <c r="B5" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C5" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="79" t="s">
+      <c r="B5" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="80" t="str">
+      <c r="E5" t="str">
         <f>IF(G5&lt;&gt;"",VLOOKUP(G5,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F5" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G5" s="79" t="s">
+      <c r="F5" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G5" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H5" s="79" t="s">
+      <c r="H5" s="23" t="s">
         <v>2077</v>
       </c>
-      <c r="I5" s="79" t="s">
+      <c r="I5" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J5" s="79"/>
-      <c r="K5" s="79" t="s">
+      <c r="J5" s="23"/>
+      <c r="K5" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L5" s="79" t="s">
+      <c r="L5" s="23" t="s">
         <v>1264</v>
       </c>
-      <c r="M5" s="79"/>
-      <c r="N5" s="79"/>
-      <c r="O5" s="79"/>
-      <c r="P5" s="79" t="s">
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q5" s="79" t="s">
+      <c r="Q5" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="79">
+      <c r="A6" s="23">
         <v>35</v>
       </c>
-      <c r="B6" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C6" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="79" t="s">
+      <c r="B6" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="80" t="str">
+      <c r="E6" t="str">
         <f>IF(G6&lt;&gt;"",VLOOKUP(G6,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F6" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G6" s="79" t="s">
+      <c r="F6" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G6" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="79" t="s">
+      <c r="H6" s="23" t="s">
         <v>2078</v>
       </c>
-      <c r="I6" s="79" t="s">
+      <c r="I6" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79" t="s">
+      <c r="J6" s="23"/>
+      <c r="K6" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L6" s="79" t="s">
+      <c r="L6" s="23" t="s">
         <v>1265</v>
       </c>
-      <c r="M6" s="79"/>
-      <c r="N6" s="79"/>
-      <c r="O6" s="79"/>
-      <c r="P6" s="79" t="s">
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q6" s="79" t="s">
+      <c r="Q6" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="79">
+      <c r="A7" s="23">
         <v>36</v>
       </c>
-      <c r="B7" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C7" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="79" t="s">
+      <c r="B7" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="80" t="str">
+      <c r="E7" t="str">
         <f>IF(G7&lt;&gt;"",VLOOKUP(G7,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F7" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G7" s="79" t="s">
+      <c r="F7" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G7" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H7" s="79" t="s">
+      <c r="H7" s="23" t="s">
         <v>2079</v>
       </c>
-      <c r="I7" s="79" t="s">
+      <c r="I7" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J7" s="79"/>
-      <c r="K7" s="79" t="s">
+      <c r="J7" s="23"/>
+      <c r="K7" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L7" s="79" t="s">
+      <c r="L7" s="23" t="s">
         <v>1266</v>
       </c>
-      <c r="M7" s="79"/>
-      <c r="N7" s="79"/>
-      <c r="O7" s="79"/>
-      <c r="P7" s="79" t="s">
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q7" s="79" t="s">
+      <c r="Q7" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="79">
+      <c r="A8" s="23">
         <v>37</v>
       </c>
-      <c r="B8" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C8" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D8" s="79" t="s">
+      <c r="B8" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="80" t="str">
+      <c r="E8" t="str">
         <f>IF(G8&lt;&gt;"",VLOOKUP(G8,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F8" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G8" s="79" t="s">
+      <c r="F8" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G8" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H8" s="79" t="s">
+      <c r="H8" s="23" t="s">
         <v>2080</v>
       </c>
-      <c r="I8" s="79" t="s">
+      <c r="I8" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79" t="s">
+      <c r="J8" s="23"/>
+      <c r="K8" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L8" s="79" t="s">
+      <c r="L8" s="23" t="s">
         <v>1267</v>
       </c>
-      <c r="M8" s="79"/>
-      <c r="N8" s="79"/>
-      <c r="O8" s="79"/>
-      <c r="P8" s="79" t="s">
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q8" s="79" t="s">
+      <c r="Q8" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="79">
+      <c r="A9" s="23">
         <v>38</v>
       </c>
-      <c r="B9" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C9" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D9" s="79" t="s">
+      <c r="B9" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="80" t="str">
+      <c r="E9" t="str">
         <f>IF(G9&lt;&gt;"",VLOOKUP(G9,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F9" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G9" s="79" t="s">
+      <c r="F9" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G9" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H9" s="79" t="s">
+      <c r="H9" s="23" t="s">
         <v>2081</v>
       </c>
-      <c r="I9" s="79" t="s">
+      <c r="I9" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J9" s="79"/>
-      <c r="K9" s="79" t="s">
+      <c r="J9" s="23"/>
+      <c r="K9" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L9" s="79" t="s">
+      <c r="L9" s="23" t="s">
         <v>1268</v>
       </c>
-      <c r="M9" s="79"/>
-      <c r="N9" s="79"/>
-      <c r="O9" s="79"/>
-      <c r="P9" s="79" t="s">
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q9" s="79" t="s">
+      <c r="Q9" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10" s="79">
+      <c r="A10" s="23">
         <v>39</v>
       </c>
-      <c r="B10" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C10" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D10" s="79" t="s">
+      <c r="B10" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="80" t="str">
+      <c r="E10" t="str">
         <f>IF(G10&lt;&gt;"",VLOOKUP(G10,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="F10" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="G10" s="79" t="s">
+      <c r="F10" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="H10" s="79" t="s">
+      <c r="H10" s="23" t="s">
         <v>2082</v>
       </c>
-      <c r="I10" s="79" t="s">
+      <c r="I10" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="J10" s="79"/>
-      <c r="K10" s="79" t="s">
+      <c r="J10" s="23"/>
+      <c r="K10" s="23" t="s">
         <v>1260</v>
       </c>
-      <c r="L10" s="79" t="s">
+      <c r="L10" s="23" t="s">
         <v>1269</v>
       </c>
-      <c r="M10" s="79"/>
-      <c r="N10" s="79"/>
-      <c r="O10" s="79"/>
-      <c r="P10" s="79" t="s">
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="23" t="s">
         <v>1270</v>
       </c>
-      <c r="Q10" s="79" t="s">
+      <c r="Q10" s="23" t="s">
         <v>1723</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="D11" s="79"/>
-      <c r="E11" s="80" t="str">
+      <c r="D11" s="23"/>
+      <c r="E11" t="str">
         <f>IF(G11&lt;&gt;"",VLOOKUP(G11,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="K11" s="79" t="s">
+      <c r="K11" s="23" t="s">
         <v>1978</v>
       </c>
-      <c r="L11" s="79" t="s">
+      <c r="L11" s="23" t="s">
         <v>1979</v>
       </c>
-      <c r="M11" s="79"/>
+      <c r="M11" s="23"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="B12" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C12" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D12" s="79"/>
-      <c r="E12" s="80" t="str">
+      <c r="B12" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" s="23"/>
+      <c r="E12" t="str">
         <f>IF(G12&lt;&gt;"",VLOOKUP(G12,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F12" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="I12" s="79" t="s">
+      <c r="F12" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="I12" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="K12" s="79" t="s">
+      <c r="K12" s="23" t="s">
         <v>2092</v>
       </c>
-      <c r="L12"/>
-      <c r="M12" s="79" t="s">
+      <c r="M12" s="23" t="s">
         <v>2091</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="B13" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="79" t="b">
-        <v>1</v>
-      </c>
-      <c r="D13" s="79"/>
-      <c r="E13" s="80" t="str">
+      <c r="B13" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" s="23"/>
+      <c r="E13" t="str">
         <f>IF(G13&lt;&gt;"",VLOOKUP(G13,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
-      <c r="F13" s="79" t="s">
-        <v>1809</v>
-      </c>
-      <c r="I13" s="79" t="s">
+      <c r="F13" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="I13" s="23" t="s">
         <v>1261</v>
       </c>
-      <c r="K13" s="79" t="s">
+      <c r="K13" s="23" t="s">
         <v>2059</v>
       </c>
-      <c r="L13"/>
-      <c r="M13" s="79" t="s">
+      <c r="M13" s="23" t="s">
         <v>2087</v>
       </c>
     </row>
@@ -55931,7 +55941,7 @@
         <v>1739</v>
       </c>
     </row>
-    <row r="68" spans="1:17" s="78" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B68" s="23" t="b">
         <v>1</v>
       </c>
@@ -55947,11 +55957,11 @@
       <c r="K68" s="23" t="s">
         <v>2055</v>
       </c>
-      <c r="M68" s="78" t="s">
+      <c r="M68" t="s">
         <v>2087</v>
       </c>
     </row>
-    <row r="69" spans="1:17" s="78" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B69" s="23" t="b">
         <v>1</v>
       </c>
@@ -55967,7 +55977,7 @@
       <c r="K69" s="23" t="s">
         <v>2058</v>
       </c>
-      <c r="M69" s="78" t="s">
+      <c r="M69" t="s">
         <v>2087</v>
       </c>
     </row>
@@ -62314,7 +62324,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{903503FA-19AE-C146-9865-7A1697985DDA}">
   <sheetPr codeName="Sheet23"/>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="28.83203125" bestFit="1" customWidth="1"/>
@@ -62326,12 +62336,13 @@
     <col min="8" max="8" width="23.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="23.1640625" customWidth="1"/>
     <col min="11" max="11" width="32.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19" customWidth="1"/>
-    <col min="13" max="13" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.6640625" customWidth="1"/>
+    <col min="12" max="12" width="32.33203125" customWidth="1"/>
+    <col min="13" max="13" width="19" customWidth="1"/>
+    <col min="14" max="14" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
@@ -62366,16 +62377,19 @@
         <v>1803</v>
       </c>
       <c r="L1" s="18" t="s">
+        <v>1791</v>
+      </c>
+      <c r="M1" s="18" t="s">
         <v>1804</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="N1" s="18" t="s">
         <v>1805</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="O1" s="18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B2" t="str">
         <f>IF(D2&lt;&gt;"",VLOOKUP(D2,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
@@ -62384,7 +62398,7 @@
         <v>1810</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="320" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" ht="320" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>1</v>
       </c>
@@ -62413,14 +62427,17 @@
       <c r="K3" t="s">
         <v>1305</v>
       </c>
-      <c r="L3" s="38" t="s">
+      <c r="L3" t="s">
+        <v>127</v>
+      </c>
+      <c r="M3" s="38" t="s">
         <v>1876</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="N3" s="38" t="s">
         <v>1877</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -62449,8 +62466,11 @@
       <c r="K4" t="s">
         <v>1474</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="304" x14ac:dyDescent="0.2">
+      <c r="L4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="304" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -62479,14 +62499,17 @@
       <c r="K5" t="s">
         <v>1479</v>
       </c>
-      <c r="L5" s="38" t="s">
+      <c r="L5" t="s">
+        <v>1115</v>
+      </c>
+      <c r="M5" s="38" t="s">
         <v>1878</v>
       </c>
-      <c r="M5" s="38" t="s">
+      <c r="N5" s="38" t="s">
         <v>1879</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="304" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" ht="304" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>1</v>
       </c>
@@ -62515,10 +62538,13 @@
       <c r="K6" t="s">
         <v>1478</v>
       </c>
-      <c r="L6" s="38" t="s">
+      <c r="L6" t="s">
+        <v>1107</v>
+      </c>
+      <c r="M6" s="38" t="s">
         <v>1880</v>
       </c>
-      <c r="M6" s="38" t="s">
+      <c r="N6" s="38" t="s">
         <v>1881</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Addition of "blank" _extra_sampleID_tag for qualityReports
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2059E499-1196-2945-ABF6-C0E11981D210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E013D3E-3AD5-6340-A899-4B406D44141F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="40720" windowHeight="20600" firstSheet="7" activeTab="14" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="40720" windowHeight="20600" firstSheet="11" activeTab="20" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="accessions_maps" sheetId="12" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9237" uniqueCount="2093">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9241" uniqueCount="2093">
   <si>
     <t>Complete</t>
   </si>
@@ -49152,7 +49152,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29B0FFD5-92F3-FD4F-93FB-9D30DA340366}">
   <sheetPr codeName="Sheet12"/>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
@@ -49700,6 +49700,31 @@
         <v>2059</v>
       </c>
       <c r="M13" s="23" t="s">
+        <v>2087</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="B14" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" s="23" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" s="23"/>
+      <c r="E14" t="str">
+        <f>IF(G14&lt;&gt;"",VLOOKUP(G14,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>1809</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>1261</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>2044</v>
+      </c>
+      <c r="M14" s="23" t="s">
         <v>2087</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove values from notes_value columns
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363CEB8E-614E-244F-A6B8-F79EC44FB5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBC2099-3C9C-2D4B-9593-D5444C5C86CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="40800" windowHeight="20740" firstSheet="13" activeTab="16" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="40800" windowHeight="20740" activeTab="3" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="accessions_maps" sheetId="12" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9398" uniqueCount="2089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9398" uniqueCount="2090">
   <si>
     <t>Complete</t>
   </si>
@@ -6412,6 +6412,9 @@
   </si>
   <si>
     <t>blank</t>
+  </si>
+  <si>
+    <t>notes_value_UNUSED</t>
   </si>
 </sst>
 </file>
@@ -6746,7 +6749,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -6900,15 +6903,9 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -32825,7 +32822,7 @@
         <v>1806</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>1791</v>
+        <v>2089</v>
       </c>
       <c r="L1" s="24" t="s">
         <v>2032</v>
@@ -33207,7 +33204,7 @@
     <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="46.6640625" customWidth="1"/>
     <col min="10" max="10" width="54.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.33203125" style="78" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="54.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -33242,7 +33239,7 @@
       <c r="J1" s="24" t="s">
         <v>2084</v>
       </c>
-      <c r="K1" s="77" t="s">
+      <c r="K1" s="24" t="s">
         <v>1784</v>
       </c>
       <c r="L1" s="24" t="s">
@@ -33272,7 +33269,7 @@
       <c r="J2" t="s">
         <v>124</v>
       </c>
-      <c r="K2" s="78" t="s">
+      <c r="K2" t="s">
         <v>2081</v>
       </c>
       <c r="L2" t="s">
@@ -33299,7 +33296,7 @@
       <c r="J3" t="s">
         <v>1991</v>
       </c>
-      <c r="K3" s="78" t="s">
+      <c r="K3" t="s">
         <v>2081</v>
       </c>
       <c r="L3" t="s">
@@ -33326,7 +33323,7 @@
       <c r="J4" t="s">
         <v>1992</v>
       </c>
-      <c r="K4" s="78" t="s">
+      <c r="K4" t="s">
         <v>2081</v>
       </c>
       <c r="L4" t="s">
@@ -33353,7 +33350,7 @@
       <c r="J5" t="s">
         <v>1993</v>
       </c>
-      <c r="K5" s="78" t="s">
+      <c r="K5" t="s">
         <v>2081</v>
       </c>
       <c r="L5" t="s">
@@ -33380,7 +33377,7 @@
       <c r="J6" t="s">
         <v>84</v>
       </c>
-      <c r="K6" s="78" t="s">
+      <c r="K6" t="s">
         <v>2081</v>
       </c>
       <c r="L6" t="s">
@@ -33407,7 +33404,7 @@
       <c r="J7" t="s">
         <v>128</v>
       </c>
-      <c r="K7" s="78" t="s">
+      <c r="K7" t="s">
         <v>2081</v>
       </c>
       <c r="L7" t="s">
@@ -33434,7 +33431,7 @@
       <c r="J8" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="78" t="s">
+      <c r="K8" t="s">
         <v>2081</v>
       </c>
       <c r="L8" t="s">
@@ -33461,7 +33458,7 @@
       <c r="J9" t="s">
         <v>15</v>
       </c>
-      <c r="K9" s="78" t="s">
+      <c r="K9" t="s">
         <v>2081</v>
       </c>
       <c r="L9" t="s">
@@ -33488,7 +33485,7 @@
       <c r="J10" t="s">
         <v>18</v>
       </c>
-      <c r="K10" s="78" t="s">
+      <c r="K10" t="s">
         <v>2081</v>
       </c>
       <c r="L10" t="s">
@@ -33515,7 +33512,7 @@
       <c r="J11" t="s">
         <v>83</v>
       </c>
-      <c r="K11" s="78" t="s">
+      <c r="K11" t="s">
         <v>2081</v>
       </c>
       <c r="L11" t="s">
@@ -33542,7 +33539,7 @@
       <c r="J12" t="s">
         <v>95</v>
       </c>
-      <c r="K12" s="78" t="s">
+      <c r="K12" t="s">
         <v>2081</v>
       </c>
       <c r="L12" t="s">
@@ -33569,7 +33566,7 @@
       <c r="J13" t="s">
         <v>1129</v>
       </c>
-      <c r="K13" s="78" t="s">
+      <c r="K13" t="s">
         <v>2081</v>
       </c>
       <c r="L13" t="s">
@@ -33596,7 +33593,7 @@
       <c r="J14" t="s">
         <v>1843</v>
       </c>
-      <c r="K14" s="78" t="s">
+      <c r="K14" t="s">
         <v>2081</v>
       </c>
       <c r="L14" t="s">
@@ -33623,7 +33620,7 @@
       <c r="J15" t="s">
         <v>125</v>
       </c>
-      <c r="K15" s="78" t="s">
+      <c r="K15" t="s">
         <v>2081</v>
       </c>
       <c r="L15" t="s">
@@ -33650,7 +33647,7 @@
       <c r="J16" t="s">
         <v>89</v>
       </c>
-      <c r="K16" s="78" t="s">
+      <c r="K16" t="s">
         <v>2081</v>
       </c>
       <c r="L16" t="s">
@@ -33677,7 +33674,7 @@
       <c r="J17" t="s">
         <v>1117</v>
       </c>
-      <c r="K17" s="78" t="s">
+      <c r="K17" t="s">
         <v>2081</v>
       </c>
       <c r="L17" t="s">
@@ -33704,7 +33701,7 @@
       <c r="J18" t="s">
         <v>91</v>
       </c>
-      <c r="K18" s="78" t="s">
+      <c r="K18" t="s">
         <v>2081</v>
       </c>
       <c r="L18" t="s">
@@ -33731,7 +33728,7 @@
       <c r="J20" t="s">
         <v>1846</v>
       </c>
-      <c r="K20" s="78" t="s">
+      <c r="K20" t="s">
         <v>2081</v>
       </c>
       <c r="L20" t="s">
@@ -33758,7 +33755,7 @@
       <c r="J22" t="s">
         <v>1122</v>
       </c>
-      <c r="K22" s="78" t="s">
+      <c r="K22" t="s">
         <v>2081</v>
       </c>
       <c r="L22" t="s">
@@ -33785,7 +33782,7 @@
       <c r="J24" t="s">
         <v>1113</v>
       </c>
-      <c r="K24" s="78" t="s">
+      <c r="K24" t="s">
         <v>2081</v>
       </c>
       <c r="L24" t="s">
@@ -33804,23 +33801,20 @@
   <dimension ref="A1:T74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="81"/>
-    <col min="2" max="2" width="39" style="81" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" style="81"/>
-    <col min="4" max="4" width="54.83203125" style="81" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="57.6640625" style="81" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.5" style="81" customWidth="1"/>
-    <col min="7" max="7" width="51" style="81" customWidth="1"/>
-    <col min="8" max="9" width="71" style="81" customWidth="1"/>
-    <col min="10" max="10" width="36.5" style="81" customWidth="1"/>
-    <col min="11" max="12" width="35.5" style="81" customWidth="1"/>
-    <col min="13" max="13" width="51" style="81" customWidth="1"/>
-    <col min="14" max="14" width="21.83203125" style="81" customWidth="1"/>
-    <col min="15" max="15" width="16.83203125" style="81" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.6640625" style="81" customWidth="1"/>
-    <col min="17" max="17" width="14.5" style="81" customWidth="1"/>
-    <col min="18" max="18" width="51" style="81" customWidth="1"/>
-    <col min="19" max="16384" width="10.83203125" style="81"/>
+    <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="54.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="57.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.5" customWidth="1"/>
+    <col min="7" max="7" width="51" customWidth="1"/>
+    <col min="8" max="9" width="71" customWidth="1"/>
+    <col min="10" max="10" width="36.5" customWidth="1"/>
+    <col min="11" max="12" width="35.5" customWidth="1"/>
+    <col min="13" max="13" width="51" customWidth="1"/>
+    <col min="14" max="14" width="21.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.6640625" customWidth="1"/>
+    <col min="17" max="17" width="14.5" customWidth="1"/>
+    <col min="18" max="18" width="51" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -33842,43 +33836,43 @@
       <c r="F1" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="79" t="s">
+      <c r="G1" s="77" t="s">
         <v>1025</v>
       </c>
-      <c r="H1" s="79" t="s">
+      <c r="H1" s="77" t="s">
         <v>1026</v>
       </c>
-      <c r="I1" s="79" t="s">
+      <c r="I1" s="77" t="s">
         <v>2068</v>
       </c>
-      <c r="J1" s="79" t="s">
+      <c r="J1" s="77" t="s">
         <v>2032</v>
       </c>
-      <c r="K1" s="79" t="s">
+      <c r="K1" s="77" t="s">
         <v>2039</v>
       </c>
-      <c r="L1" s="79" t="s">
+      <c r="L1" s="77" t="s">
         <v>2085</v>
       </c>
-      <c r="M1" s="79" t="s">
+      <c r="M1" s="77" t="s">
         <v>2022</v>
       </c>
-      <c r="N1" s="79" t="s">
+      <c r="N1" s="77" t="s">
         <v>1985</v>
       </c>
-      <c r="O1" s="79" t="s">
+      <c r="O1" s="77" t="s">
         <v>2023</v>
       </c>
-      <c r="P1" s="79" t="s">
+      <c r="P1" s="77" t="s">
         <v>1703</v>
       </c>
-      <c r="Q1" s="79" t="s">
+      <c r="Q1" s="77" t="s">
         <v>1699</v>
       </c>
-      <c r="R1" s="79" t="s">
+      <c r="R1" s="77" t="s">
         <v>1700</v>
       </c>
-      <c r="S1" s="80" t="s">
+      <c r="S1" s="78" t="s">
         <v>9</v>
       </c>
       <c r="T1" s="17" t="s">
@@ -33886,3084 +33880,3084 @@
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A2" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B2" s="81" t="str">
+      <c r="A2" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
         <f>IF(D2&lt;&gt;"",VLOOKUP(D2,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C2" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D2" s="82" t="s">
+      <c r="C2" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E2" s="82" t="s">
+      <c r="E2" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="F2" s="82" t="s">
+      <c r="F2" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G2" s="82" t="s">
+      <c r="G2" s="6" t="s">
         <v>1215</v>
       </c>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82" t="s">
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K2" s="82" t="s">
+      <c r="K2" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L2" s="82" t="s">
+      <c r="L2" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M2" s="82" t="s">
+      <c r="M2" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82" t="s">
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q2" s="82" t="s">
+      <c r="Q2" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R2" s="82" t="s">
+      <c r="R2" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S2" s="82"/>
+      <c r="S2" s="6"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A3" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B3" s="81" t="str">
+      <c r="A3" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" t="str">
         <f>IF(D3&lt;&gt;"",VLOOKUP(D3,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C3" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D3" s="82" t="s">
+      <c r="C3" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E3" s="82" t="s">
+      <c r="E3" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F3" s="82" t="s">
+      <c r="F3" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G3" s="82" t="s">
+      <c r="G3" s="6" t="s">
         <v>1216</v>
       </c>
-      <c r="H3" s="82"/>
-      <c r="I3" s="82"/>
-      <c r="J3" s="82" t="s">
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K3" s="82" t="s">
+      <c r="K3" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L3" s="82" t="s">
+      <c r="L3" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M3" s="82" t="s">
+      <c r="M3" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N3" s="82"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82" t="s">
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q3" s="82" t="s">
+      <c r="Q3" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R3" s="82" t="s">
+      <c r="R3" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S3" s="82"/>
+      <c r="S3" s="6"/>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A4" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B4" s="81" t="str">
+      <c r="A4" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" t="str">
         <f>IF(D4&lt;&gt;"",VLOOKUP(D4,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C4" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D4" s="82" t="s">
+      <c r="C4" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E4" s="82" t="s">
+      <c r="E4" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="F4" s="82" t="s">
+      <c r="F4" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G4" s="82" t="s">
+      <c r="G4" s="6" t="s">
         <v>1235</v>
       </c>
-      <c r="H4" s="82"/>
-      <c r="I4" s="82"/>
-      <c r="J4" s="82" t="s">
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K4" s="82" t="s">
+      <c r="K4" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L4" s="82" t="s">
+      <c r="L4" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M4" s="82" t="s">
+      <c r="M4" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N4" s="82"/>
-      <c r="O4" s="82"/>
-      <c r="P4" s="82" t="s">
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q4" s="82" t="s">
+      <c r="Q4" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R4" s="82" t="s">
+      <c r="R4" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S4" s="82"/>
+      <c r="S4" s="6"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A5" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" s="81" t="str">
+      <c r="A5" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" t="str">
         <f>IF(D5&lt;&gt;"",VLOOKUP(D5,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C5" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D5" s="82" t="s">
+      <c r="C5" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E5" s="82" t="s">
+      <c r="E5" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="F5" s="82" t="s">
+      <c r="F5" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G5" s="82" t="s">
+      <c r="G5" s="6" t="s">
         <v>1236</v>
       </c>
-      <c r="H5" s="82"/>
-      <c r="I5" s="82"/>
-      <c r="J5" s="82" t="s">
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K5" s="82" t="s">
+      <c r="K5" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L5" s="82" t="s">
+      <c r="L5" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M5" s="82" t="s">
+      <c r="M5" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N5" s="82"/>
-      <c r="O5" s="82"/>
-      <c r="P5" s="82" t="s">
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q5" s="82" t="s">
+      <c r="Q5" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R5" s="82" t="s">
+      <c r="R5" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S5" s="82"/>
+      <c r="S5" s="6"/>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A6" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B6" s="81" t="str">
+      <c r="A6" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" t="str">
         <f>IF(D6&lt;&gt;"",VLOOKUP(D6,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C6" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D6" s="82" t="s">
+      <c r="C6" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="82" t="s">
+      <c r="E6" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="F6" s="82" t="s">
+      <c r="F6" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G6" s="82" t="s">
+      <c r="G6" s="6" t="s">
         <v>1217</v>
       </c>
-      <c r="H6" s="82"/>
-      <c r="I6" s="82"/>
-      <c r="J6" s="82" t="s">
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K6" s="82" t="s">
+      <c r="K6" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L6" s="82" t="s">
+      <c r="L6" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M6" s="82" t="s">
+      <c r="M6" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N6" s="82"/>
-      <c r="O6" s="82"/>
-      <c r="P6" s="82" t="s">
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q6" s="82" t="s">
+      <c r="Q6" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R6" s="82" t="s">
+      <c r="R6" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S6" s="82"/>
+      <c r="S6" s="6"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B7" s="81" t="str">
+      <c r="A7" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B7" t="str">
         <f>IF(D7&lt;&gt;"",VLOOKUP(D7,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C7" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D7" s="82" t="s">
+      <c r="C7" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="82" t="s">
+      <c r="E7" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="F7" s="82" t="s">
+      <c r="F7" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G7" s="82" t="s">
+      <c r="G7" s="6" t="s">
         <v>1218</v>
       </c>
-      <c r="H7" s="82"/>
-      <c r="I7" s="82"/>
-      <c r="J7" s="82" t="s">
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K7" s="82" t="s">
+      <c r="K7" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L7" s="82" t="s">
+      <c r="L7" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M7" s="82" t="s">
+      <c r="M7" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N7" s="82"/>
-      <c r="O7" s="82"/>
-      <c r="P7" s="82" t="s">
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q7" s="82" t="s">
+      <c r="Q7" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R7" s="82" t="s">
+      <c r="R7" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S7" s="82"/>
+      <c r="S7" s="6"/>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A8" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B8" s="81" t="str">
+      <c r="A8" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" t="str">
         <f>IF(D8&lt;&gt;"",VLOOKUP(D8,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C8" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D8" s="82" t="s">
+      <c r="C8" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E8" s="82" t="s">
+      <c r="E8" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="F8" s="82" t="s">
+      <c r="F8" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G8" s="82" t="s">
+      <c r="G8" s="6" t="s">
         <v>1219</v>
       </c>
-      <c r="H8" s="82"/>
-      <c r="I8" s="82"/>
-      <c r="J8" s="82" t="s">
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K8" s="82" t="s">
+      <c r="K8" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L8" s="82" t="s">
+      <c r="L8" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M8" s="82" t="s">
+      <c r="M8" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N8" s="82"/>
-      <c r="O8" s="82"/>
-      <c r="P8" s="82" t="s">
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q8" s="82" t="s">
+      <c r="Q8" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R8" s="82" t="s">
+      <c r="R8" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S8" s="82"/>
+      <c r="S8" s="6"/>
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" s="81" t="str">
+      <c r="A9" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" t="str">
         <f>IF(D9&lt;&gt;"",VLOOKUP(D9,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C9" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D9" s="82" t="s">
+      <c r="C9" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E9" s="82" t="s">
+      <c r="E9" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="F9" s="82" t="s">
+      <c r="F9" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G9" s="82" t="s">
+      <c r="G9" s="6" t="s">
         <v>1220</v>
       </c>
-      <c r="H9" s="82"/>
-      <c r="I9" s="82"/>
-      <c r="J9" s="82" t="s">
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K9" s="82" t="s">
+      <c r="K9" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L9" s="82" t="s">
+      <c r="L9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M9" s="82" t="s">
+      <c r="M9" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N9" s="82"/>
-      <c r="O9" s="82"/>
-      <c r="P9" s="82" t="s">
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q9" s="82" t="s">
+      <c r="Q9" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R9" s="82" t="s">
+      <c r="R9" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S9" s="82"/>
+      <c r="S9" s="6"/>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A10" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" s="81" t="str">
+      <c r="A10" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="str">
         <f>IF(D10&lt;&gt;"",VLOOKUP(D10,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C10" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D10" s="82" t="s">
+      <c r="C10" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="82" t="s">
+      <c r="E10" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="F10" s="82" t="s">
+      <c r="F10" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G10" s="82" t="s">
+      <c r="G10" s="6" t="s">
         <v>1221</v>
       </c>
-      <c r="H10" s="82"/>
-      <c r="I10" s="82"/>
-      <c r="J10" s="82" t="s">
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K10" s="82" t="s">
+      <c r="K10" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L10" s="82" t="s">
+      <c r="L10" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M10" s="82" t="s">
+      <c r="M10" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N10" s="82"/>
-      <c r="O10" s="82"/>
-      <c r="P10" s="82" t="s">
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q10" s="82" t="s">
+      <c r="Q10" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R10" s="82" t="s">
+      <c r="R10" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S10" s="82"/>
+      <c r="S10" s="6"/>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A11" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B11" s="81" t="str">
+      <c r="A11" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" t="str">
         <f>IF(D11&lt;&gt;"",VLOOKUP(D11,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C11" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D11" s="82" t="s">
+      <c r="C11" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E11" s="82" t="s">
+      <c r="E11" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="F11" s="82" t="s">
+      <c r="F11" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G11" s="82" t="s">
+      <c r="G11" s="6" t="s">
         <v>1222</v>
       </c>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
-      <c r="J11" s="82" t="s">
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K11" s="82" t="s">
+      <c r="K11" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L11" s="82" t="s">
+      <c r="L11" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M11" s="82" t="s">
+      <c r="M11" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N11" s="82"/>
-      <c r="O11" s="82"/>
-      <c r="P11" s="82" t="s">
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q11" s="82" t="s">
+      <c r="Q11" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R11" s="82" t="s">
+      <c r="R11" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S11" s="82"/>
+      <c r="S11" s="6"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A12" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" s="81" t="str">
+      <c r="A12" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" t="str">
         <f>IF(D12&lt;&gt;"",VLOOKUP(D12,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C12" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D12" s="82" t="s">
+      <c r="C12" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E12" s="82" t="s">
+      <c r="E12" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="F12" s="82" t="s">
+      <c r="F12" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G12" s="82" t="s">
+      <c r="G12" s="6" t="s">
         <v>1223</v>
       </c>
-      <c r="H12" s="82"/>
-      <c r="I12" s="82"/>
-      <c r="J12" s="82" t="s">
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K12" s="82" t="s">
+      <c r="K12" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L12" s="82" t="s">
+      <c r="L12" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M12" s="82" t="s">
+      <c r="M12" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N12" s="82"/>
-      <c r="O12" s="82"/>
-      <c r="P12" s="82" t="s">
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q12" s="82" t="s">
+      <c r="Q12" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R12" s="82" t="s">
+      <c r="R12" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S12" s="82"/>
+      <c r="S12" s="6"/>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A13" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B13" s="81" t="str">
+      <c r="A13" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" t="str">
         <f>IF(D13&lt;&gt;"",VLOOKUP(D13,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C13" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D13" s="82" t="s">
+      <c r="C13" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E13" s="82" t="s">
+      <c r="E13" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="F13" s="82" t="s">
+      <c r="F13" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G13" s="82" t="s">
+      <c r="G13" s="6" t="s">
         <v>1224</v>
       </c>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
-      <c r="J13" s="82" t="s">
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K13" s="82" t="s">
+      <c r="K13" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L13" s="82" t="s">
+      <c r="L13" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M13" s="82" t="s">
+      <c r="M13" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N13" s="82"/>
-      <c r="O13" s="82"/>
-      <c r="P13" s="82" t="s">
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q13" s="82" t="s">
+      <c r="Q13" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R13" s="82" t="s">
+      <c r="R13" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S13" s="82"/>
+      <c r="S13" s="6"/>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A14" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" s="81" t="str">
+      <c r="A14" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" t="str">
         <f>IF(D14&lt;&gt;"",VLOOKUP(D14,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C14" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D14" s="82" t="s">
+      <c r="C14" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D14" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E14" s="82" t="s">
+      <c r="E14" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="F14" s="82" t="s">
+      <c r="F14" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G14" s="82" t="s">
+      <c r="G14" s="6" t="s">
         <v>1225</v>
       </c>
-      <c r="H14" s="82"/>
-      <c r="I14" s="82"/>
-      <c r="J14" s="82" t="s">
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K14" s="82" t="s">
+      <c r="K14" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L14" s="82" t="s">
+      <c r="L14" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M14" s="82" t="s">
+      <c r="M14" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N14" s="82"/>
-      <c r="O14" s="82"/>
-      <c r="P14" s="82" t="s">
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q14" s="82" t="s">
+      <c r="Q14" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R14" s="82" t="s">
+      <c r="R14" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S14" s="82"/>
+      <c r="S14" s="6"/>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A15" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" s="81" t="str">
+      <c r="A15" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="str">
         <f>IF(D15&lt;&gt;"",VLOOKUP(D15,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C15" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D15" s="82" t="s">
+      <c r="C15" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E15" s="82" t="s">
+      <c r="E15" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="F15" s="82" t="s">
+      <c r="F15" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G15" s="82" t="s">
+      <c r="G15" s="6" t="s">
         <v>1226</v>
       </c>
-      <c r="H15" s="82"/>
-      <c r="I15" s="82"/>
-      <c r="J15" s="82" t="s">
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K15" s="82" t="s">
+      <c r="K15" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L15" s="82" t="s">
+      <c r="L15" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M15" s="82" t="s">
+      <c r="M15" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N15" s="82"/>
-      <c r="O15" s="82"/>
-      <c r="P15" s="82" t="s">
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q15" s="82" t="s">
+      <c r="Q15" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R15" s="82" t="s">
+      <c r="R15" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S15" s="82"/>
+      <c r="S15" s="6"/>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A16" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" s="81" t="str">
+      <c r="A16" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="str">
         <f>IF(D16&lt;&gt;"",VLOOKUP(D16,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C16" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D16" s="82" t="s">
+      <c r="C16" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E16" s="82" t="s">
+      <c r="E16" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="F16" s="82" t="s">
+      <c r="F16" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G16" s="82" t="s">
+      <c r="G16" s="6" t="s">
         <v>1227</v>
       </c>
-      <c r="H16" s="82"/>
-      <c r="I16" s="82"/>
-      <c r="J16" s="82" t="s">
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K16" s="82" t="s">
+      <c r="K16" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L16" s="82" t="s">
+      <c r="L16" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M16" s="82" t="s">
+      <c r="M16" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N16" s="82"/>
-      <c r="O16" s="82"/>
-      <c r="P16" s="82" t="s">
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q16" s="82" t="s">
+      <c r="Q16" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R16" s="82" t="s">
+      <c r="R16" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S16" s="82"/>
+      <c r="S16" s="6"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A17" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" s="81" t="str">
+      <c r="A17" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="str">
         <f>IF(D17&lt;&gt;"",VLOOKUP(D17,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C17" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D17" s="82" t="s">
+      <c r="C17" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E17" s="82" t="s">
+      <c r="E17" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="F17" s="82" t="s">
+      <c r="F17" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G17" s="82" t="s">
+      <c r="G17" s="6" t="s">
         <v>1228</v>
       </c>
-      <c r="H17" s="82"/>
-      <c r="I17" s="82"/>
-      <c r="J17" s="82" t="s">
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K17" s="82" t="s">
+      <c r="K17" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L17" s="82" t="s">
+      <c r="L17" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M17" s="82" t="s">
+      <c r="M17" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N17" s="82"/>
-      <c r="O17" s="82"/>
-      <c r="P17" s="82" t="s">
+      <c r="N17" s="6"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q17" s="82" t="s">
+      <c r="Q17" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R17" s="82" t="s">
+      <c r="R17" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S17" s="82"/>
+      <c r="S17" s="6"/>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" s="81" t="str">
+      <c r="A18" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" t="str">
         <f>IF(D18&lt;&gt;"",VLOOKUP(D18,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C18" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D18" s="82" t="s">
+      <c r="C18" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E18" s="82" t="s">
+      <c r="E18" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="F18" s="82" t="s">
+      <c r="F18" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G18" s="82" t="s">
+      <c r="G18" s="6" t="s">
         <v>1229</v>
       </c>
-      <c r="H18" s="82"/>
-      <c r="I18" s="82"/>
-      <c r="J18" s="82" t="s">
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K18" s="82" t="s">
+      <c r="K18" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L18" s="82" t="s">
+      <c r="L18" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M18" s="82" t="s">
+      <c r="M18" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N18" s="82"/>
-      <c r="O18" s="82"/>
-      <c r="P18" s="82" t="s">
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q18" s="82" t="s">
+      <c r="Q18" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R18" s="82" t="s">
+      <c r="R18" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S18" s="82"/>
+      <c r="S18" s="6"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B19" s="81" t="str">
+      <c r="A19" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" t="str">
         <f>IF(D19&lt;&gt;"",VLOOKUP(D19,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C19" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D19" s="82" t="s">
+      <c r="C19" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E19" s="82" t="s">
+      <c r="E19" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="F19" s="82" t="s">
+      <c r="F19" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G19" s="82" t="s">
+      <c r="G19" s="6" t="s">
         <v>1230</v>
       </c>
-      <c r="H19" s="82"/>
-      <c r="I19" s="82"/>
-      <c r="J19" s="82" t="s">
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K19" s="82" t="s">
+      <c r="K19" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L19" s="82" t="s">
+      <c r="L19" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M19" s="82" t="s">
+      <c r="M19" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N19" s="82"/>
-      <c r="O19" s="82"/>
-      <c r="P19" s="82" t="s">
+      <c r="N19" s="6"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q19" s="82" t="s">
+      <c r="Q19" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R19" s="82" t="s">
+      <c r="R19" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S19" s="82"/>
+      <c r="S19" s="6"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A20" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B20" s="81" t="str">
+      <c r="A20" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" t="str">
         <f>IF(D20&lt;&gt;"",VLOOKUP(D20,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C20" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D20" s="82" t="s">
+      <c r="C20" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D20" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E20" s="82" t="s">
+      <c r="E20" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="F20" s="82" t="s">
+      <c r="F20" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G20" s="82" t="s">
+      <c r="G20" s="6" t="s">
         <v>1231</v>
       </c>
-      <c r="H20" s="82"/>
-      <c r="I20" s="82"/>
-      <c r="J20" s="82" t="s">
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K20" s="82" t="s">
+      <c r="K20" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L20" s="82" t="s">
+      <c r="L20" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M20" s="82" t="s">
+      <c r="M20" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N20" s="82"/>
-      <c r="O20" s="82"/>
-      <c r="P20" s="82" t="s">
+      <c r="N20" s="6"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q20" s="82" t="s">
+      <c r="Q20" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R20" s="82" t="s">
+      <c r="R20" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S20" s="82"/>
+      <c r="S20" s="6"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A21" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B21" s="81" t="str">
+      <c r="A21" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" t="str">
         <f>IF(D21&lt;&gt;"",VLOOKUP(D21,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C21" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D21" s="82" t="s">
+      <c r="C21" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E21" s="82" t="s">
+      <c r="E21" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="F21" s="82" t="s">
+      <c r="F21" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G21" s="82" t="s">
+      <c r="G21" s="6" t="s">
         <v>1232</v>
       </c>
-      <c r="H21" s="82"/>
-      <c r="I21" s="82"/>
-      <c r="J21" s="82" t="s">
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K21" s="82" t="s">
+      <c r="K21" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L21" s="82" t="s">
+      <c r="L21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M21" s="82" t="s">
+      <c r="M21" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N21" s="82"/>
-      <c r="O21" s="82"/>
-      <c r="P21" s="82" t="s">
+      <c r="N21" s="6"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q21" s="82" t="s">
+      <c r="Q21" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R21" s="82" t="s">
+      <c r="R21" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S21" s="82"/>
+      <c r="S21" s="6"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B22" s="81" t="str">
+      <c r="A22" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" t="str">
         <f>IF(D22&lt;&gt;"",VLOOKUP(D22,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C22" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D22" s="82" t="s">
+      <c r="C22" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E22" s="82" t="s">
+      <c r="E22" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="F22" s="82" t="s">
+      <c r="F22" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G22" s="82" t="s">
+      <c r="G22" s="6" t="s">
         <v>1233</v>
       </c>
-      <c r="H22" s="82"/>
-      <c r="I22" s="82"/>
-      <c r="J22" s="82" t="s">
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K22" s="82" t="s">
+      <c r="K22" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L22" s="82" t="s">
+      <c r="L22" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M22" s="82" t="s">
+      <c r="M22" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N22" s="82"/>
-      <c r="O22" s="82"/>
-      <c r="P22" s="82" t="s">
+      <c r="N22" s="6"/>
+      <c r="O22" s="6"/>
+      <c r="P22" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q22" s="82" t="s">
+      <c r="Q22" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R22" s="82" t="s">
+      <c r="R22" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S22" s="82"/>
+      <c r="S22" s="6"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B23" s="81" t="str">
+      <c r="A23" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" t="str">
         <f>IF(D23&lt;&gt;"",VLOOKUP(D23,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C23" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D23" s="82" t="s">
+      <c r="C23" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="E23" s="82" t="s">
+      <c r="E23" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="F23" s="82" t="s">
+      <c r="F23" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G23" s="82" t="s">
+      <c r="G23" s="6" t="s">
         <v>1234</v>
       </c>
-      <c r="H23" s="82"/>
-      <c r="I23" s="82"/>
-      <c r="J23" s="82" t="s">
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K23" s="82" t="s">
+      <c r="K23" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L23" s="82" t="s">
+      <c r="L23" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="M23" s="82" t="s">
+      <c r="M23" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N23" s="82"/>
-      <c r="O23" s="82"/>
-      <c r="P23" s="82" t="s">
+      <c r="N23" s="6"/>
+      <c r="O23" s="6"/>
+      <c r="P23" s="6" t="s">
         <v>1087</v>
       </c>
-      <c r="Q23" s="82" t="s">
+      <c r="Q23" s="6" t="s">
         <v>1238</v>
       </c>
-      <c r="R23" s="82" t="s">
+      <c r="R23" s="6" t="s">
         <v>1698</v>
       </c>
-      <c r="S23" s="82"/>
+      <c r="S23" s="6"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B24" s="81" t="str">
+      <c r="B24" t="str">
         <f>IF(D24&lt;&gt;"",VLOOKUP(D24,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B25" s="81" t="str">
+      <c r="A25" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B25" t="str">
         <f>IF(D25&lt;&gt;"",VLOOKUP(D25,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Environmental conditions and measurements</v>
       </c>
-      <c r="C25" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D25" s="82" t="s">
+      <c r="C25" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>1846</v>
       </c>
-      <c r="E25" s="82"/>
-      <c r="F25" s="82" t="s">
+      <c r="E25" s="6"/>
+      <c r="F25" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G25" s="82"/>
-      <c r="H25" s="82"/>
-      <c r="I25" s="82"/>
-      <c r="J25" s="82" t="s">
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K25" s="82" t="s">
+      <c r="K25" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L25" s="82" t="s">
+      <c r="L25" s="6" t="s">
         <v>1846</v>
       </c>
-      <c r="M25" s="82" t="s">
+      <c r="M25" s="6" t="s">
         <v>1988</v>
       </c>
-      <c r="N25" s="82"/>
-      <c r="O25" s="82"/>
-      <c r="P25" s="82"/>
-      <c r="Q25" s="82" t="s">
+      <c r="N25" s="6"/>
+      <c r="O25" s="6"/>
+      <c r="P25" s="6"/>
+      <c r="Q25" s="6" t="s">
         <v>1396</v>
       </c>
-      <c r="R25" s="82" t="s">
+      <c r="R25" s="6" t="s">
         <v>1865</v>
       </c>
-      <c r="S25" s="83" t="s">
+      <c r="S25" s="5" t="s">
         <v>1397</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B26" s="81" t="str">
+      <c r="B26" t="str">
         <f>IF(D26&lt;&gt;"",VLOOKUP(D26,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B27" s="81" t="e">
+      <c r="A27" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B27" t="e">
         <f>IF(D27&lt;&gt;"",VLOOKUP(D27,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C27" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D27" s="82" t="s">
+      <c r="C27" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="E27" s="82" t="s">
+      <c r="E27" s="6" t="s">
         <v>1999</v>
       </c>
-      <c r="F27" s="82" t="s">
+      <c r="F27" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G27" s="82" t="s">
+      <c r="G27" s="6" t="s">
         <v>1412</v>
       </c>
-      <c r="H27" s="82"/>
-      <c r="I27" s="82"/>
-      <c r="J27" s="82"/>
-      <c r="K27" s="82"/>
-      <c r="L27" s="82" t="s">
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="M27" s="82" t="s">
+      <c r="M27" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N27" s="82"/>
-      <c r="O27" s="82"/>
-      <c r="P27" s="82"/>
-      <c r="Q27" s="82" t="s">
+      <c r="N27" s="6"/>
+      <c r="O27" s="6"/>
+      <c r="P27" s="6"/>
+      <c r="Q27" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R27" s="82" t="s">
+      <c r="R27" s="6" t="s">
         <v>1994</v>
       </c>
-      <c r="S27" s="82"/>
+      <c r="S27" s="6"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A28" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B28" s="81" t="e">
+      <c r="A28" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B28" t="e">
         <f>IF(D28&lt;&gt;"",VLOOKUP(D28,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C28" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D28" s="82" t="s">
+      <c r="C28" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="E28" s="82" t="s">
+      <c r="E28" s="6" t="s">
         <v>1998</v>
       </c>
-      <c r="F28" s="82" t="s">
+      <c r="F28" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G28" s="82" t="s">
+      <c r="G28" s="6" t="s">
         <v>1413</v>
       </c>
-      <c r="H28" s="82"/>
-      <c r="I28" s="82"/>
-      <c r="J28" s="82"/>
-      <c r="K28" s="82"/>
-      <c r="L28" s="82" t="s">
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="M28" s="82" t="s">
+      <c r="M28" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N28" s="82"/>
-      <c r="O28" s="82"/>
-      <c r="P28" s="82"/>
-      <c r="Q28" s="82" t="s">
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R28" s="82" t="s">
+      <c r="R28" s="6" t="s">
         <v>1994</v>
       </c>
-      <c r="S28" s="82"/>
+      <c r="S28" s="6"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A29" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B29" s="81" t="e">
+      <c r="A29" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B29" t="e">
         <f>IF(D29&lt;&gt;"",VLOOKUP(D29,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C29" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D29" s="82" t="s">
+      <c r="C29" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D29" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="E29" s="82" t="s">
+      <c r="E29" s="6" t="s">
         <v>1997</v>
       </c>
-      <c r="F29" s="82" t="s">
+      <c r="F29" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G29" s="82" t="s">
+      <c r="G29" s="6" t="s">
         <v>1415</v>
       </c>
-      <c r="H29" s="82"/>
-      <c r="I29" s="82"/>
-      <c r="J29" s="82"/>
-      <c r="K29" s="82"/>
-      <c r="L29" s="82" t="s">
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6" t="s">
         <v>1991</v>
       </c>
-      <c r="M29" s="82" t="s">
+      <c r="M29" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N29" s="82"/>
-      <c r="O29" s="82"/>
-      <c r="P29" s="82"/>
-      <c r="Q29" s="82" t="s">
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6" t="s">
         <v>1416</v>
       </c>
-      <c r="R29" s="82" t="s">
+      <c r="R29" s="6" t="s">
         <v>1994</v>
       </c>
-      <c r="S29" s="82"/>
+      <c r="S29" s="6"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B30" s="81" t="str">
+      <c r="B30" t="str">
         <f>IF(D30&lt;&gt;"",VLOOKUP(D30,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A31" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B31" s="81" t="e">
+      <c r="A31" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B31" t="e">
         <f>IF(D31&lt;&gt;"",VLOOKUP(D31,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C31" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D31" s="82" t="s">
+      <c r="C31" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="E31" s="82" t="s">
+      <c r="E31" s="6" t="s">
         <v>1999</v>
       </c>
-      <c r="F31" s="82" t="s">
+      <c r="F31" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G31" s="82" t="s">
+      <c r="G31" s="6" t="s">
         <v>1412</v>
       </c>
-      <c r="H31" s="82"/>
-      <c r="I31" s="82"/>
-      <c r="J31" s="82"/>
-      <c r="K31" s="82"/>
-      <c r="L31" s="82" t="s">
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="6"/>
+      <c r="K31" s="6"/>
+      <c r="L31" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="M31" s="82" t="s">
+      <c r="M31" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N31" s="82"/>
-      <c r="O31" s="82"/>
-      <c r="P31" s="82"/>
-      <c r="Q31" s="82" t="s">
+      <c r="N31" s="6"/>
+      <c r="O31" s="6"/>
+      <c r="P31" s="6"/>
+      <c r="Q31" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R31" s="82" t="s">
+      <c r="R31" s="6" t="s">
         <v>1995</v>
       </c>
-      <c r="S31" s="82"/>
+      <c r="S31" s="6"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A32" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B32" s="81" t="e">
+      <c r="A32" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B32" t="e">
         <f>IF(D32&lt;&gt;"",VLOOKUP(D32,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C32" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D32" s="82" t="s">
+      <c r="C32" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="E32" s="82" t="s">
+      <c r="E32" s="6" t="s">
         <v>1998</v>
       </c>
-      <c r="F32" s="82" t="s">
+      <c r="F32" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G32" s="82" t="s">
+      <c r="G32" s="6" t="s">
         <v>1413</v>
       </c>
-      <c r="H32" s="82"/>
-      <c r="I32" s="82"/>
-      <c r="J32" s="82"/>
-      <c r="K32" s="82"/>
-      <c r="L32" s="82" t="s">
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="6"/>
+      <c r="L32" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="M32" s="82" t="s">
+      <c r="M32" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N32" s="82"/>
-      <c r="O32" s="82"/>
-      <c r="P32" s="82"/>
-      <c r="Q32" s="82" t="s">
+      <c r="N32" s="6"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="6"/>
+      <c r="Q32" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R32" s="82" t="s">
+      <c r="R32" s="6" t="s">
         <v>1995</v>
       </c>
-      <c r="S32" s="82"/>
+      <c r="S32" s="6"/>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A33" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B33" s="81" t="e">
+      <c r="A33" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B33" t="e">
         <f>IF(D33&lt;&gt;"",VLOOKUP(D33,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C33" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D33" s="82" t="s">
+      <c r="C33" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="E33" s="82" t="s">
+      <c r="E33" s="6" t="s">
         <v>1997</v>
       </c>
-      <c r="F33" s="82" t="s">
+      <c r="F33" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G33" s="82" t="s">
+      <c r="G33" s="6" t="s">
         <v>1415</v>
       </c>
-      <c r="H33" s="82"/>
-      <c r="I33" s="82"/>
-      <c r="J33" s="82"/>
-      <c r="K33" s="82"/>
-      <c r="L33" s="82" t="s">
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="6"/>
+      <c r="L33" s="6" t="s">
         <v>1992</v>
       </c>
-      <c r="M33" s="82" t="s">
+      <c r="M33" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N33" s="82"/>
-      <c r="O33" s="82"/>
-      <c r="P33" s="82"/>
-      <c r="Q33" s="82" t="s">
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6" t="s">
         <v>1416</v>
       </c>
-      <c r="R33" s="82" t="s">
+      <c r="R33" s="6" t="s">
         <v>1995</v>
       </c>
-      <c r="S33" s="82"/>
+      <c r="S33" s="6"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B34" s="81" t="str">
+      <c r="B34" t="str">
         <f>IF(D34&lt;&gt;"",VLOOKUP(D34,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A35" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B35" s="81" t="e">
+      <c r="A35" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B35" t="e">
         <f>IF(D35&lt;&gt;"",VLOOKUP(D35,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C35" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D35" s="82" t="s">
+      <c r="C35" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="E35" s="82" t="s">
+      <c r="E35" s="6" t="s">
         <v>1999</v>
       </c>
-      <c r="F35" s="82" t="s">
+      <c r="F35" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G35" s="82" t="s">
+      <c r="G35" s="6" t="s">
         <v>1412</v>
       </c>
-      <c r="H35" s="82"/>
-      <c r="I35" s="82"/>
-      <c r="J35" s="82"/>
-      <c r="K35" s="82"/>
-      <c r="L35" s="82" t="s">
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="6"/>
+      <c r="L35" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="M35" s="82" t="s">
+      <c r="M35" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N35" s="82"/>
-      <c r="O35" s="82"/>
-      <c r="P35" s="82"/>
-      <c r="Q35" s="82" t="s">
+      <c r="N35" s="6"/>
+      <c r="O35" s="6"/>
+      <c r="P35" s="6"/>
+      <c r="Q35" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R35" s="82" t="s">
+      <c r="R35" s="6" t="s">
         <v>1996</v>
       </c>
-      <c r="S35" s="82"/>
+      <c r="S35" s="6"/>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A36" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B36" s="81" t="e">
+      <c r="A36" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B36" t="e">
         <f>IF(D36&lt;&gt;"",VLOOKUP(D36,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C36" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D36" s="82" t="s">
+      <c r="C36" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="E36" s="82" t="s">
+      <c r="E36" s="6" t="s">
         <v>1998</v>
       </c>
-      <c r="F36" s="82" t="s">
+      <c r="F36" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G36" s="82" t="s">
+      <c r="G36" s="6" t="s">
         <v>1413</v>
       </c>
-      <c r="H36" s="82"/>
-      <c r="I36" s="82"/>
-      <c r="J36" s="82"/>
-      <c r="K36" s="82"/>
-      <c r="L36" s="82" t="s">
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="6"/>
+      <c r="K36" s="6"/>
+      <c r="L36" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="M36" s="82" t="s">
+      <c r="M36" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N36" s="82"/>
-      <c r="O36" s="82"/>
-      <c r="P36" s="82"/>
-      <c r="Q36" s="82" t="s">
+      <c r="N36" s="6"/>
+      <c r="O36" s="6"/>
+      <c r="P36" s="6"/>
+      <c r="Q36" s="6" t="s">
         <v>1414</v>
       </c>
-      <c r="R36" s="82" t="s">
+      <c r="R36" s="6" t="s">
         <v>1996</v>
       </c>
-      <c r="S36" s="82"/>
+      <c r="S36" s="6"/>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A37" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B37" s="81" t="e">
+      <c r="A37" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B37" t="e">
         <f>IF(D37&lt;&gt;"",VLOOKUP(D37,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>#N/A</v>
       </c>
-      <c r="C37" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D37" s="82" t="s">
+      <c r="C37" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="E37" s="82" t="s">
+      <c r="E37" s="6" t="s">
         <v>1997</v>
       </c>
-      <c r="F37" s="82" t="s">
+      <c r="F37" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G37" s="82" t="s">
+      <c r="G37" s="6" t="s">
         <v>1415</v>
       </c>
-      <c r="H37" s="82"/>
-      <c r="I37" s="82"/>
-      <c r="J37" s="82"/>
-      <c r="K37" s="82"/>
-      <c r="L37" s="82" t="s">
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6" t="s">
         <v>1993</v>
       </c>
-      <c r="M37" s="82" t="s">
+      <c r="M37" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N37" s="82"/>
-      <c r="O37" s="82"/>
-      <c r="P37" s="82"/>
-      <c r="Q37" s="82" t="s">
+      <c r="N37" s="6"/>
+      <c r="O37" s="6"/>
+      <c r="P37" s="6"/>
+      <c r="Q37" s="6" t="s">
         <v>1416</v>
       </c>
-      <c r="R37" s="82" t="s">
+      <c r="R37" s="6" t="s">
         <v>1996</v>
       </c>
-      <c r="S37" s="82"/>
+      <c r="S37" s="6"/>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B38" s="81" t="str">
+      <c r="B38" t="str">
         <f>IF(D38&lt;&gt;"",VLOOKUP(D38,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="39" spans="1:20" s="24" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="86" t="b">
+      <c r="A39" s="80" t="b">
         <v>0</v>
       </c>
       <c r="B39" s="24" t="str">
         <f>IF(D39&lt;&gt;"",VLOOKUP(D39,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C39" s="86" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D39" s="86" t="s">
+      <c r="C39" s="80" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D39" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="E39" s="86" t="s">
+      <c r="E39" s="80" t="s">
         <v>1159</v>
       </c>
-      <c r="F39" s="86" t="s">
+      <c r="F39" s="80" t="s">
         <v>1237</v>
       </c>
-      <c r="G39" s="86" t="s">
+      <c r="G39" s="80" t="s">
         <v>1487</v>
       </c>
-      <c r="H39" s="86" t="s">
+      <c r="H39" s="80" t="s">
         <v>1740</v>
       </c>
-      <c r="I39" s="86"/>
-      <c r="J39" s="86" t="s">
+      <c r="I39" s="80"/>
+      <c r="J39" s="80" t="s">
         <v>1115</v>
       </c>
-      <c r="K39" s="86" t="s">
+      <c r="K39" s="80" t="s">
         <v>1115</v>
       </c>
-      <c r="L39" s="86" t="s">
+      <c r="L39" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="M39" s="86" t="s">
+      <c r="M39" s="80" t="s">
         <v>2075</v>
       </c>
-      <c r="N39" s="86"/>
-      <c r="O39" s="86" t="s">
+      <c r="N39" s="80"/>
+      <c r="O39" s="80" t="s">
         <v>1037</v>
       </c>
-      <c r="P39" s="86"/>
-      <c r="Q39" s="86" t="s">
+      <c r="P39" s="80"/>
+      <c r="Q39" s="80" t="s">
         <v>1489</v>
       </c>
-      <c r="R39" s="86" t="s">
+      <c r="R39" s="80" t="s">
         <v>1705</v>
       </c>
-      <c r="S39" s="86"/>
-      <c r="T39" s="86" t="s">
+      <c r="S39" s="80"/>
+      <c r="T39" s="80" t="s">
         <v>2000</v>
       </c>
     </row>
     <row r="40" spans="1:20" s="24" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="86" t="b">
+      <c r="A40" s="80" t="b">
         <v>0</v>
       </c>
       <c r="B40" s="24" t="str">
         <f>IF(D40&lt;&gt;"",VLOOKUP(D40,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C40" s="86" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D40" s="86" t="s">
+      <c r="C40" s="80" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D40" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="E40" s="86" t="s">
+      <c r="E40" s="80" t="s">
         <v>1160</v>
       </c>
-      <c r="F40" s="86" t="s">
+      <c r="F40" s="80" t="s">
         <v>1237</v>
       </c>
-      <c r="G40" s="86" t="s">
+      <c r="G40" s="80" t="s">
         <v>1488</v>
       </c>
-      <c r="H40" s="86" t="s">
+      <c r="H40" s="80" t="s">
         <v>1740</v>
       </c>
-      <c r="I40" s="86"/>
-      <c r="J40" s="86" t="s">
+      <c r="I40" s="80"/>
+      <c r="J40" s="80" t="s">
         <v>1115</v>
       </c>
-      <c r="K40" s="86" t="s">
+      <c r="K40" s="80" t="s">
         <v>1115</v>
       </c>
-      <c r="L40" s="86" t="s">
+      <c r="L40" s="80" t="s">
         <v>84</v>
       </c>
-      <c r="M40" s="86" t="s">
+      <c r="M40" s="80" t="s">
         <v>2075</v>
       </c>
-      <c r="N40" s="86"/>
-      <c r="O40" s="86" t="s">
+      <c r="N40" s="80"/>
+      <c r="O40" s="80" t="s">
         <v>1037</v>
       </c>
-      <c r="P40" s="86"/>
-      <c r="Q40" s="86" t="s">
+      <c r="P40" s="80"/>
+      <c r="Q40" s="80" t="s">
         <v>1489</v>
       </c>
-      <c r="R40" s="86" t="s">
+      <c r="R40" s="80" t="s">
         <v>1705</v>
       </c>
-      <c r="S40" s="86"/>
-      <c r="T40" s="86" t="s">
+      <c r="S40" s="80"/>
+      <c r="T40" s="80" t="s">
         <v>2000</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B41" s="81" t="str">
+      <c r="B41" t="str">
         <f>IF(D41&lt;&gt;"",VLOOKUP(D41,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A42" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B42" s="81" t="str">
+      <c r="A42" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B42" t="str">
         <f>IF(D42&lt;&gt;"",VLOOKUP(D42,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C42" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D42" s="82" t="s">
+      <c r="C42" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E42" s="82" t="s">
+      <c r="E42" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="F42" s="82" t="s">
+      <c r="F42" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G42" s="82" t="s">
+      <c r="G42" s="6" t="s">
         <v>1538</v>
       </c>
-      <c r="H42" s="82"/>
-      <c r="I42" s="82"/>
-      <c r="J42" s="82" t="s">
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K42" s="82" t="s">
+      <c r="K42" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L42" s="82" t="s">
+      <c r="L42" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M42" s="82" t="s">
+      <c r="M42" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N42" s="82" t="s">
+      <c r="N42" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O42" s="82" t="s">
+      <c r="O42" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P42" s="82"/>
+      <c r="P42" s="6"/>
       <c r="Q42" s="12" t="s">
         <v>1538</v>
       </c>
       <c r="R42" s="12" t="s">
         <v>759</v>
       </c>
-      <c r="S42" s="83" t="s">
+      <c r="S42" s="5" t="s">
         <v>1549</v>
       </c>
-      <c r="T42" s="81" t="s">
+      <c r="T42" t="s">
         <v>1539</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A43" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B43" s="81" t="str">
+      <c r="A43" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B43" t="str">
         <f>IF(D43&lt;&gt;"",VLOOKUP(D43,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C43" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D43" s="82" t="s">
+      <c r="C43" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E43" s="82" t="s">
+      <c r="E43" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F43" s="82" t="s">
+      <c r="F43" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G43" s="82" t="s">
+      <c r="G43" s="6" t="s">
         <v>1542</v>
       </c>
-      <c r="H43" s="82"/>
-      <c r="I43" s="82"/>
-      <c r="J43" s="82" t="s">
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K43" s="82" t="s">
+      <c r="K43" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L43" s="82" t="s">
+      <c r="L43" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M43" s="82" t="s">
+      <c r="M43" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N43" s="82" t="s">
+      <c r="N43" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O43" s="82" t="s">
+      <c r="O43" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P43" s="82"/>
+      <c r="P43" s="6"/>
       <c r="Q43" s="12" t="s">
         <v>1542</v>
       </c>
       <c r="R43" s="12" t="s">
         <v>1543</v>
       </c>
-      <c r="S43" s="83" t="s">
+      <c r="S43" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A44" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B44" s="81" t="str">
+      <c r="A44" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B44" t="str">
         <f>IF(D44&lt;&gt;"",VLOOKUP(D44,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C44" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D44" s="82" t="s">
+      <c r="C44" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E44" s="82" t="s">
+      <c r="E44" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="F44" s="82" t="s">
+      <c r="F44" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G44" s="82" t="s">
+      <c r="G44" s="6" t="s">
         <v>1542</v>
       </c>
-      <c r="H44" s="82"/>
-      <c r="I44" s="82"/>
-      <c r="J44" s="82" t="s">
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K44" s="82" t="s">
+      <c r="K44" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L44" s="82" t="s">
+      <c r="L44" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M44" s="82" t="s">
+      <c r="M44" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N44" s="82" t="s">
+      <c r="N44" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O44" s="82" t="s">
+      <c r="O44" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P44" s="82"/>
+      <c r="P44" s="6"/>
       <c r="Q44" s="12" t="s">
         <v>1542</v>
       </c>
       <c r="R44" s="12" t="s">
         <v>1544</v>
       </c>
-      <c r="S44" s="83" t="s">
+      <c r="S44" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A45" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B45" s="81" t="str">
+      <c r="A45" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B45" t="str">
         <f>IF(D45&lt;&gt;"",VLOOKUP(D45,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C45" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D45" s="82" t="s">
+      <c r="C45" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E45" s="82" t="s">
+      <c r="E45" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F45" s="82" t="s">
+      <c r="F45" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G45" s="82" t="s">
+      <c r="G45" s="6" t="s">
         <v>1538</v>
       </c>
-      <c r="H45" s="82"/>
-      <c r="I45" s="82"/>
-      <c r="J45" s="82" t="s">
+      <c r="H45" s="6"/>
+      <c r="I45" s="6"/>
+      <c r="J45" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K45" s="82" t="s">
+      <c r="K45" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L45" s="82" t="s">
+      <c r="L45" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M45" s="82" t="s">
+      <c r="M45" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N45" s="82" t="s">
+      <c r="N45" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O45" s="82" t="s">
+      <c r="O45" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P45" s="82"/>
+      <c r="P45" s="6"/>
       <c r="Q45" s="12" t="s">
         <v>1538</v>
       </c>
       <c r="R45" s="12" t="s">
         <v>1545</v>
       </c>
-      <c r="S45" s="83" t="s">
+      <c r="S45" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A46" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B46" s="81" t="str">
+      <c r="A46" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B46" t="str">
         <f>IF(D46&lt;&gt;"",VLOOKUP(D46,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C46" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D46" s="82" t="s">
+      <c r="C46" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E46" s="82" t="s">
+      <c r="E46" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="F46" s="82" t="s">
+      <c r="F46" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G46" s="82" t="s">
+      <c r="G46" s="6" t="s">
         <v>1538</v>
       </c>
-      <c r="H46" s="82"/>
-      <c r="I46" s="82"/>
-      <c r="J46" s="82" t="s">
+      <c r="H46" s="6"/>
+      <c r="I46" s="6"/>
+      <c r="J46" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K46" s="82" t="s">
+      <c r="K46" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L46" s="82" t="s">
+      <c r="L46" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M46" s="82" t="s">
+      <c r="M46" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N46" s="82" t="s">
+      <c r="N46" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O46" s="82" t="s">
+      <c r="O46" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P46" s="82"/>
+      <c r="P46" s="6"/>
       <c r="Q46" s="12" t="s">
         <v>1538</v>
       </c>
       <c r="R46" s="12" t="s">
         <v>1546</v>
       </c>
-      <c r="S46" s="83" t="s">
+      <c r="S46" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A47" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B47" s="81" t="str">
+      <c r="A47" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B47" t="str">
         <f>IF(D47&lt;&gt;"",VLOOKUP(D47,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C47" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D47" s="82" t="s">
+      <c r="C47" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E47" s="82" t="s">
+      <c r="E47" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="F47" s="82" t="s">
+      <c r="F47" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G47" s="82" t="s">
+      <c r="G47" s="6" t="s">
         <v>1538</v>
       </c>
-      <c r="H47" s="82"/>
-      <c r="I47" s="82"/>
-      <c r="J47" s="82" t="s">
+      <c r="H47" s="6"/>
+      <c r="I47" s="6"/>
+      <c r="J47" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K47" s="82" t="s">
+      <c r="K47" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L47" s="82" t="s">
+      <c r="L47" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M47" s="82" t="s">
+      <c r="M47" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N47" s="82" t="s">
+      <c r="N47" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O47" s="82" t="s">
+      <c r="O47" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P47" s="82"/>
+      <c r="P47" s="6"/>
       <c r="Q47" s="12" t="s">
         <v>1538</v>
       </c>
       <c r="R47" s="12" t="s">
         <v>1547</v>
       </c>
-      <c r="S47" s="83" t="s">
+      <c r="S47" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A48" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B48" s="81" t="str">
+      <c r="A48" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B48" t="str">
         <f>IF(D48&lt;&gt;"",VLOOKUP(D48,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C48" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D48" s="82" t="s">
+      <c r="C48" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E48" s="82" t="s">
+      <c r="E48" s="6" t="s">
         <v>2005</v>
       </c>
-      <c r="F48" s="82" t="s">
+      <c r="F48" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G48" s="82" t="s">
+      <c r="G48" s="6" t="s">
         <v>1542</v>
       </c>
-      <c r="H48" s="82"/>
-      <c r="I48" s="82"/>
-      <c r="J48" s="82" t="s">
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K48" s="82" t="s">
+      <c r="K48" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L48" s="82" t="s">
+      <c r="L48" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M48" s="82" t="s">
+      <c r="M48" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N48" s="82" t="s">
+      <c r="N48" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O48" s="82" t="s">
+      <c r="O48" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P48" s="82"/>
+      <c r="P48" s="6"/>
       <c r="Q48" s="12" t="s">
         <v>1542</v>
       </c>
       <c r="R48" s="12" t="s">
         <v>1548</v>
       </c>
-      <c r="S48" s="83" t="s">
+      <c r="S48" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A49" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B49" s="81" t="str">
+      <c r="A49" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B49" t="str">
         <f>IF(D49&lt;&gt;"",VLOOKUP(D49,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C49" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D49" s="82" t="s">
+      <c r="C49" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E49" s="82" t="s">
+      <c r="E49" s="6" t="s">
         <v>1136</v>
       </c>
-      <c r="F49" s="82" t="s">
+      <c r="F49" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G49" s="84" t="s">
+      <c r="G49" s="79" t="s">
         <v>1416</v>
       </c>
-      <c r="H49" s="82"/>
-      <c r="I49" s="82"/>
-      <c r="J49" s="82" t="s">
+      <c r="H49" s="6"/>
+      <c r="I49" s="6"/>
+      <c r="J49" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K49" s="82" t="s">
+      <c r="K49" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L49" s="82" t="s">
+      <c r="L49" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M49" s="82" t="s">
+      <c r="M49" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N49" s="82" t="s">
+      <c r="N49" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O49" s="82" t="s">
+      <c r="O49" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P49" s="82"/>
+      <c r="P49" s="6"/>
       <c r="Q49" s="13" t="s">
         <v>1416</v>
       </c>
       <c r="R49" s="14" t="s">
         <v>1550</v>
       </c>
-      <c r="S49" s="83" t="s">
+      <c r="S49" s="5" t="s">
         <v>1549</v>
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A50" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B50" s="81" t="str">
+      <c r="A50" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B50" t="str">
         <f>IF(D50&lt;&gt;"",VLOOKUP(D50,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C50" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D50" s="82" t="s">
+      <c r="C50" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E50" s="82" t="s">
+      <c r="E50" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="F50" s="82" t="s">
+      <c r="F50" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G50" s="82" t="s">
+      <c r="G50" s="6" t="s">
         <v>1540</v>
       </c>
-      <c r="H50" s="82"/>
-      <c r="I50" s="82"/>
-      <c r="J50" s="82" t="s">
+      <c r="H50" s="6"/>
+      <c r="I50" s="6"/>
+      <c r="J50" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K50" s="82" t="s">
+      <c r="K50" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L50" s="82" t="s">
+      <c r="L50" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="M50" s="82" t="s">
+      <c r="M50" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N50" s="82" t="s">
+      <c r="N50" s="6" t="s">
         <v>1536</v>
       </c>
-      <c r="O50" s="82" t="s">
+      <c r="O50" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P50" s="82"/>
+      <c r="P50" s="6"/>
       <c r="Q50" s="12" t="s">
         <v>1540</v>
       </c>
       <c r="R50" s="12" t="b">
         <v>1</v>
       </c>
-      <c r="S50" s="83" t="s">
+      <c r="S50" s="5" t="s">
         <v>1549</v>
       </c>
-      <c r="T50" s="81" t="s">
+      <c r="T50" t="s">
         <v>1541</v>
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B51" s="81" t="str">
+      <c r="B51" t="str">
         <f>IF(D51&lt;&gt;"",VLOOKUP(D51,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A52" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B52" s="81" t="str">
+      <c r="A52" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B52" t="str">
         <f>IF(D52&lt;&gt;"",VLOOKUP(D52,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>AMR detection information</v>
       </c>
-      <c r="C52" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D52" s="82" t="s">
+      <c r="C52" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D52" s="6" t="s">
         <v>1122</v>
       </c>
-      <c r="E52" s="82"/>
-      <c r="F52" s="82" t="s">
+      <c r="E52" s="6"/>
+      <c r="F52" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G52" s="82"/>
-      <c r="H52" s="82" t="s">
+      <c r="G52" s="6"/>
+      <c r="H52" s="6" t="s">
         <v>1718</v>
       </c>
-      <c r="I52" s="82"/>
-      <c r="J52" s="82" t="s">
+      <c r="I52" s="6"/>
+      <c r="J52" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K52" s="82" t="s">
+      <c r="K52" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L52" s="82" t="s">
+      <c r="L52" s="6" t="s">
         <v>1122</v>
       </c>
-      <c r="M52" s="82" t="s">
+      <c r="M52" s="6" t="s">
         <v>2076</v>
       </c>
-      <c r="N52" s="82"/>
-      <c r="O52" s="82" t="s">
+      <c r="N52" s="6"/>
+      <c r="O52" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P52" s="82"/>
-      <c r="Q52" s="82" t="s">
+      <c r="P52" s="6"/>
+      <c r="Q52" s="6" t="s">
         <v>1567</v>
       </c>
-      <c r="R52" s="82" t="s">
+      <c r="R52" s="6" t="s">
         <v>1686</v>
       </c>
-      <c r="S52" s="83" t="s">
+      <c r="S52" s="5" t="s">
         <v>1568</v>
       </c>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A53" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B53" s="81" t="str">
+      <c r="A53" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B53" t="str">
         <f>IF(D53&lt;&gt;"",VLOOKUP(D53,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="C53" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D53" s="82" t="s">
+      <c r="C53" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E53" s="82"/>
-      <c r="F53" s="82" t="s">
+      <c r="E53" s="6"/>
+      <c r="F53" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G53" s="82"/>
-      <c r="H53" s="82" t="s">
+      <c r="G53" s="6"/>
+      <c r="H53" s="6" t="s">
         <v>1715</v>
       </c>
-      <c r="I53" s="82"/>
-      <c r="J53" s="82" t="s">
+      <c r="I53" s="6"/>
+      <c r="J53" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K53" s="82" t="s">
+      <c r="K53" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L53" s="82" t="s">
+      <c r="L53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="M53" s="82" t="s">
+      <c r="M53" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N53" s="82"/>
-      <c r="O53" s="82" t="s">
+      <c r="N53" s="6"/>
+      <c r="O53" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P53" s="82"/>
-      <c r="Q53" s="82" t="s">
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6" t="s">
         <v>1571</v>
       </c>
-      <c r="R53" s="82" t="s">
+      <c r="R53" s="6" t="s">
         <v>1687</v>
       </c>
-      <c r="S53" s="83" t="s">
+      <c r="S53" s="5" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A54" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B54" s="81" t="str">
+      <c r="A54" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B54" t="str">
         <f>IF(D54&lt;&gt;"",VLOOKUP(D54,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="C54" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D54" s="82" t="s">
+      <c r="C54" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D54" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E54" s="82"/>
-      <c r="F54" s="82" t="s">
+      <c r="E54" s="6"/>
+      <c r="F54" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G54" s="82"/>
-      <c r="H54" s="82"/>
-      <c r="I54" s="82"/>
-      <c r="J54" s="82" t="s">
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K54" s="82" t="s">
+      <c r="K54" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L54" s="82" t="s">
+      <c r="L54" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="M54" s="82" t="s">
+      <c r="M54" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N54" s="82"/>
-      <c r="O54" s="82" t="s">
+      <c r="N54" s="6"/>
+      <c r="O54" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P54" s="82"/>
-      <c r="Q54" s="82" t="s">
+      <c r="P54" s="6"/>
+      <c r="Q54" s="6" t="s">
         <v>1574</v>
       </c>
-      <c r="R54" s="82" t="s">
+      <c r="R54" s="6" t="s">
         <v>1688</v>
       </c>
-      <c r="S54" s="83" t="s">
+      <c r="S54" s="5" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A55" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B55" s="81" t="str">
+      <c r="A55" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B55" t="str">
         <f>IF(D55&lt;&gt;"",VLOOKUP(D55,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="C55" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D55" s="82" t="s">
+      <c r="C55" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E55" s="82"/>
-      <c r="F55" s="82" t="s">
+      <c r="E55" s="6"/>
+      <c r="F55" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G55" s="82"/>
-      <c r="H55" s="82"/>
-      <c r="I55" s="82"/>
-      <c r="J55" s="82" t="s">
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K55" s="82" t="s">
+      <c r="K55" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L55" s="82" t="s">
+      <c r="L55" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="M55" s="82" t="s">
+      <c r="M55" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N55" s="82"/>
-      <c r="O55" s="82" t="s">
+      <c r="N55" s="6"/>
+      <c r="O55" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P55" s="82"/>
-      <c r="Q55" s="82" t="s">
+      <c r="P55" s="6"/>
+      <c r="Q55" s="6" t="s">
         <v>1575</v>
       </c>
-      <c r="R55" s="82" t="s">
+      <c r="R55" s="6" t="s">
         <v>1689</v>
       </c>
-      <c r="S55" s="83" t="s">
+      <c r="S55" s="5" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="56" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A56" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B56" s="81" t="str">
+      <c r="A56" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B56" t="str">
         <f>IF(D56&lt;&gt;"",VLOOKUP(D56,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="C56" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D56" s="82" t="s">
+      <c r="C56" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E56" s="82"/>
-      <c r="F56" s="82" t="s">
+      <c r="E56" s="6"/>
+      <c r="F56" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G56" s="82"/>
-      <c r="H56" s="82"/>
-      <c r="I56" s="82"/>
-      <c r="J56" s="82" t="s">
+      <c r="G56" s="6"/>
+      <c r="H56" s="6"/>
+      <c r="I56" s="6"/>
+      <c r="J56" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K56" s="82" t="s">
+      <c r="K56" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L56" s="82" t="s">
+      <c r="L56" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="M56" s="82" t="s">
+      <c r="M56" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N56" s="82"/>
-      <c r="O56" s="82" t="s">
+      <c r="N56" s="6"/>
+      <c r="O56" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P56" s="82"/>
-      <c r="Q56" s="82" t="s">
+      <c r="P56" s="6"/>
+      <c r="Q56" s="6" t="s">
         <v>1579</v>
       </c>
-      <c r="R56" s="82" t="s">
+      <c r="R56" s="6" t="s">
         <v>1690</v>
       </c>
-      <c r="S56" s="83" t="s">
+      <c r="S56" s="5" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A57" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B57" s="81" t="str">
+      <c r="A57" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B57" t="str">
         <f>IF(D57&lt;&gt;"",VLOOKUP(D57,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Bioinformatics and QC metrics</v>
       </c>
-      <c r="C57" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D57" s="82" t="s">
+      <c r="C57" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="E57" s="82"/>
-      <c r="F57" s="82" t="s">
+      <c r="E57" s="6"/>
+      <c r="F57" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G57" s="82"/>
-      <c r="H57" s="82" t="s">
+      <c r="G57" s="6"/>
+      <c r="H57" s="6" t="s">
         <v>1716</v>
       </c>
-      <c r="I57" s="82"/>
-      <c r="J57" s="82" t="s">
+      <c r="I57" s="6"/>
+      <c r="J57" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K57" s="82" t="s">
+      <c r="K57" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L57" s="82" t="s">
+      <c r="L57" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="M57" s="82" t="s">
+      <c r="M57" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N57" s="82"/>
-      <c r="O57" s="82" t="s">
+      <c r="N57" s="6"/>
+      <c r="O57" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P57" s="82"/>
-      <c r="Q57" s="82" t="s">
+      <c r="P57" s="6"/>
+      <c r="Q57" s="6" t="s">
         <v>1581</v>
       </c>
-      <c r="R57" s="82" t="s">
+      <c r="R57" s="6" t="s">
         <v>1691</v>
       </c>
-      <c r="S57" s="83" t="s">
+      <c r="S57" s="5" t="s">
         <v>1572</v>
       </c>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A58" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B58" s="81" t="str">
+      <c r="A58" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B58" t="str">
         <f>IF(D58&lt;&gt;"",VLOOKUP(D58,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Lineage/clade information</v>
       </c>
-      <c r="C58" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D58" s="82" t="s">
+      <c r="C58" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D58" s="6" t="s">
         <v>1129</v>
       </c>
-      <c r="E58" s="82"/>
-      <c r="F58" s="82" t="s">
+      <c r="E58" s="6"/>
+      <c r="F58" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G58" s="82"/>
-      <c r="H58" s="82"/>
-      <c r="I58" s="82"/>
-      <c r="J58" s="82" t="s">
+      <c r="G58" s="6"/>
+      <c r="H58" s="6"/>
+      <c r="I58" s="6"/>
+      <c r="J58" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K58" s="82" t="s">
+      <c r="K58" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L58" s="82" t="s">
+      <c r="L58" s="6" t="s">
         <v>1129</v>
       </c>
-      <c r="M58" s="82" t="s">
+      <c r="M58" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N58" s="82"/>
-      <c r="O58" s="82" t="s">
+      <c r="N58" s="6"/>
+      <c r="O58" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P58" s="82"/>
-      <c r="Q58" s="82" t="s">
+      <c r="P58" s="6"/>
+      <c r="Q58" s="6" t="s">
         <v>1583</v>
       </c>
-      <c r="R58" s="82" t="s">
+      <c r="R58" s="6" t="s">
         <v>1692</v>
       </c>
-      <c r="S58" s="83" t="s">
+      <c r="S58" s="5" t="s">
         <v>1584</v>
       </c>
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B59" s="81" t="str">
+      <c r="B59" t="str">
         <f>IF(D59&lt;&gt;"",VLOOKUP(D59,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A60" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B60" s="81" t="str">
+      <c r="A60" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B60" t="str">
         <f>IF(D60&lt;&gt;"",VLOOKUP(D60,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C60" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D60" s="82" t="s">
+      <c r="C60" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D60" s="6" t="s">
         <v>1843</v>
       </c>
-      <c r="E60" s="82"/>
-      <c r="F60" s="82" t="s">
+      <c r="E60" s="6"/>
+      <c r="F60" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G60" s="82"/>
-      <c r="H60" s="82" t="s">
+      <c r="G60" s="6"/>
+      <c r="H60" s="6" t="s">
         <v>2018</v>
       </c>
-      <c r="I60" s="82"/>
-      <c r="J60" s="82" t="s">
+      <c r="I60" s="6"/>
+      <c r="J60" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K60" s="82" t="s">
+      <c r="K60" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L60" s="82" t="s">
+      <c r="L60" s="6" t="s">
         <v>1843</v>
       </c>
-      <c r="M60" s="82" t="s">
+      <c r="M60" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N60" s="82"/>
-      <c r="O60" s="82" t="s">
+      <c r="N60" s="6"/>
+      <c r="O60" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P60" s="82"/>
-      <c r="Q60" s="82" t="s">
+      <c r="P60" s="6"/>
+      <c r="Q60" s="6" t="s">
         <v>1593</v>
       </c>
-      <c r="R60" s="82" t="s">
+      <c r="R60" s="6" t="s">
         <v>2019</v>
       </c>
-      <c r="S60" s="83" t="s">
+      <c r="S60" s="5" t="s">
         <v>1594</v>
       </c>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B61" s="81" t="str">
+      <c r="B61" t="str">
         <f>IF(D61&lt;&gt;"",VLOOKUP(D61,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A62" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B62" s="81" t="str">
+      <c r="A62" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B62" t="str">
         <f>IF(D62&lt;&gt;"",VLOOKUP(D62,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sample collection and processing</v>
       </c>
-      <c r="C62" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D62" s="82" t="s">
+      <c r="C62" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="E62" s="82"/>
-      <c r="F62" s="82" t="s">
+      <c r="E62" s="6"/>
+      <c r="F62" s="6" t="s">
         <v>1237</v>
       </c>
       <c r="G62" s="9"/>
-      <c r="H62" s="82" t="s">
+      <c r="H62" s="6" t="s">
         <v>1738</v>
       </c>
-      <c r="I62" s="82"/>
-      <c r="J62" s="82" t="s">
+      <c r="I62" s="6"/>
+      <c r="J62" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="K62" s="82" t="s">
+      <c r="K62" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="L62" s="82" t="s">
+      <c r="L62" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="M62" s="82" t="s">
+      <c r="M62" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N62" s="82"/>
-      <c r="O62" s="82" t="s">
+      <c r="N62" s="6"/>
+      <c r="O62" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P62" s="82"/>
-      <c r="Q62" s="82" t="s">
+      <c r="P62" s="6"/>
+      <c r="Q62" s="6" t="s">
         <v>1606</v>
       </c>
-      <c r="R62" s="82" t="s">
+      <c r="R62" s="6" t="s">
         <v>1605</v>
       </c>
-      <c r="S62" s="83" t="s">
+      <c r="S62" s="5" t="s">
         <v>1607</v>
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="B63" s="81" t="str">
+      <c r="B63" t="str">
         <f>IF(D63&lt;&gt;"",VLOOKUP(D63,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A64" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B64" s="81" t="str">
+      <c r="A64" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B64" t="str">
         <f>IF(D64&lt;&gt;"",VLOOKUP(D64,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C64" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D64" s="82" t="s">
+      <c r="C64" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D64" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E64" s="82"/>
-      <c r="F64" s="82" t="s">
+      <c r="E64" s="6"/>
+      <c r="F64" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G64" s="82"/>
-      <c r="H64" s="82" t="s">
+      <c r="G64" s="6"/>
+      <c r="H64" s="6" t="s">
         <v>1741</v>
       </c>
-      <c r="I64" s="82"/>
-      <c r="J64" s="82" t="s">
+      <c r="I64" s="6"/>
+      <c r="J64" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K64" s="82" t="s">
+      <c r="K64" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L64" s="82" t="s">
+      <c r="L64" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="M64" s="82" t="s">
+      <c r="M64" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N64" s="82"/>
-      <c r="O64" s="82" t="s">
+      <c r="N64" s="6"/>
+      <c r="O64" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P64" s="82"/>
-      <c r="Q64" s="82" t="s">
+      <c r="P64" s="6"/>
+      <c r="Q64" s="6" t="s">
         <v>1619</v>
       </c>
-      <c r="R64" s="82" t="s">
+      <c r="R64" s="6" t="s">
         <v>1618</v>
       </c>
-      <c r="S64" s="83" t="s">
+      <c r="S64" s="5" t="s">
         <v>1620</v>
       </c>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B65" s="81" t="str">
+      <c r="B65" t="str">
         <f>IF(D65&lt;&gt;"",VLOOKUP(D65,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="66" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A66" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B66" s="81" t="str">
+      <c r="A66" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B66" t="str">
         <f>IF(D66&lt;&gt;"",VLOOKUP(D66,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C66" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D66" s="82" t="s">
+      <c r="C66" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D66" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E66" s="82" t="s">
+      <c r="E66" s="6" t="s">
         <v>2004</v>
       </c>
-      <c r="F66" s="82" t="s">
+      <c r="F66" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G66" s="82" t="s">
+      <c r="G66" s="6" t="s">
         <v>1624</v>
       </c>
-      <c r="H66" s="82"/>
-      <c r="I66" s="82" t="s">
+      <c r="H66" s="6"/>
+      <c r="I66" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J66" s="82" t="s">
+      <c r="J66" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K66" s="82" t="s">
+      <c r="K66" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L66" s="82" t="s">
+      <c r="L66" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="M66" s="82" t="s">
+      <c r="M66" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N66" s="82"/>
-      <c r="O66" s="82" t="s">
+      <c r="N66" s="6"/>
+      <c r="O66" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P66" s="82"/>
-      <c r="Q66" s="82" t="s">
+      <c r="P66" s="6"/>
+      <c r="Q66" s="6" t="s">
         <v>1622</v>
       </c>
-      <c r="R66" s="82" t="s">
+      <c r="R66" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="S66" s="83" t="s">
+      <c r="S66" s="5" t="s">
         <v>1629</v>
       </c>
     </row>
     <row r="67" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A67" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B67" s="81" t="str">
+      <c r="A67" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B67" t="str">
         <f>IF(D67&lt;&gt;"",VLOOKUP(D67,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C67" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D67" s="82" t="s">
+      <c r="C67" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D67" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E67" s="82" t="s">
+      <c r="E67" s="6" t="s">
         <v>1623</v>
       </c>
-      <c r="F67" s="82" t="s">
+      <c r="F67" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G67" s="82" t="s">
+      <c r="G67" s="6" t="s">
         <v>1626</v>
       </c>
-      <c r="H67" s="82"/>
-      <c r="I67" s="82" t="s">
+      <c r="H67" s="6"/>
+      <c r="I67" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J67" s="82" t="s">
+      <c r="J67" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K67" s="82" t="s">
+      <c r="K67" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L67" s="82" t="s">
+      <c r="L67" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="M67" s="82" t="s">
+      <c r="M67" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N67" s="82"/>
-      <c r="O67" s="82" t="s">
+      <c r="N67" s="6"/>
+      <c r="O67" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P67" s="82"/>
-      <c r="Q67" s="82" t="s">
+      <c r="P67" s="6"/>
+      <c r="Q67" s="6" t="s">
         <v>1622</v>
       </c>
-      <c r="R67" s="82" t="s">
+      <c r="R67" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="S67" s="83" t="s">
+      <c r="S67" s="5" t="s">
         <v>1629</v>
       </c>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A68" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B68" s="81" t="str">
+      <c r="A68" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B68" t="str">
         <f>IF(D68&lt;&gt;"",VLOOKUP(D68,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C68" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D68" s="82" t="s">
+      <c r="C68" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E68" s="82" t="s">
+      <c r="E68" s="6" t="s">
         <v>2003</v>
       </c>
-      <c r="F68" s="82" t="s">
+      <c r="F68" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G68" s="82" t="s">
+      <c r="G68" s="6" t="s">
         <v>1625</v>
       </c>
-      <c r="H68" s="82"/>
-      <c r="I68" s="82" t="s">
+      <c r="H68" s="6"/>
+      <c r="I68" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J68" s="82" t="s">
+      <c r="J68" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K68" s="82" t="s">
+      <c r="K68" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L68" s="82" t="s">
+      <c r="L68" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="M68" s="82" t="s">
+      <c r="M68" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N68" s="82"/>
-      <c r="O68" s="82" t="s">
+      <c r="N68" s="6"/>
+      <c r="O68" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P68" s="82"/>
-      <c r="Q68" s="82" t="s">
+      <c r="P68" s="6"/>
+      <c r="Q68" s="6" t="s">
         <v>1622</v>
       </c>
-      <c r="R68" s="82" t="s">
+      <c r="R68" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="S68" s="83" t="s">
+      <c r="S68" s="5" t="s">
         <v>1629</v>
       </c>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A69" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B69" s="81" t="str">
+      <c r="A69" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B69" t="str">
         <f>IF(D69&lt;&gt;"",VLOOKUP(D69,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C69" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D69" s="82" t="s">
+      <c r="C69" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D69" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E69" s="82" t="s">
+      <c r="E69" s="6" t="s">
         <v>2001</v>
       </c>
-      <c r="F69" s="82" t="s">
+      <c r="F69" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G69" s="82" t="s">
+      <c r="G69" s="6" t="s">
         <v>1627</v>
       </c>
-      <c r="H69" s="82"/>
-      <c r="I69" s="82" t="s">
+      <c r="H69" s="6"/>
+      <c r="I69" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J69" s="82" t="s">
+      <c r="J69" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K69" s="82" t="s">
+      <c r="K69" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L69" s="82" t="s">
+      <c r="L69" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="M69" s="82" t="s">
+      <c r="M69" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N69" s="82"/>
-      <c r="O69" s="82" t="s">
+      <c r="N69" s="6"/>
+      <c r="O69" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P69" s="82"/>
-      <c r="Q69" s="82" t="s">
+      <c r="P69" s="6"/>
+      <c r="Q69" s="6" t="s">
         <v>1622</v>
       </c>
-      <c r="R69" s="82" t="s">
+      <c r="R69" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="S69" s="83" t="s">
+      <c r="S69" s="5" t="s">
         <v>1629</v>
       </c>
     </row>
     <row r="70" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A70" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B70" s="81" t="str">
+      <c r="A70" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B70" t="str">
         <f>IF(D70&lt;&gt;"",VLOOKUP(D70,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Sequence information</v>
       </c>
-      <c r="C70" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D70" s="82" t="s">
+      <c r="C70" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D70" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="E70" s="82" t="s">
+      <c r="E70" s="6" t="s">
         <v>2002</v>
       </c>
-      <c r="F70" s="82" t="s">
+      <c r="F70" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G70" s="82" t="s">
+      <c r="G70" s="6" t="s">
         <v>1628</v>
       </c>
-      <c r="H70" s="82"/>
-      <c r="I70" s="82" t="s">
+      <c r="H70" s="6"/>
+      <c r="I70" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J70" s="82" t="s">
+      <c r="J70" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K70" s="82" t="s">
+      <c r="K70" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L70" s="82" t="s">
+      <c r="L70" s="6" t="s">
         <v>1117</v>
       </c>
-      <c r="M70" s="82" t="s">
+      <c r="M70" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N70" s="82"/>
-      <c r="O70" s="82" t="s">
+      <c r="N70" s="6"/>
+      <c r="O70" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P70" s="82"/>
-      <c r="Q70" s="82" t="s">
+      <c r="P70" s="6"/>
+      <c r="Q70" s="6" t="s">
         <v>1622</v>
       </c>
-      <c r="R70" s="82" t="s">
+      <c r="R70" s="6" t="s">
         <v>1714</v>
       </c>
-      <c r="S70" s="83" t="s">
+      <c r="S70" s="5" t="s">
         <v>1629</v>
       </c>
     </row>
     <row r="71" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B71" s="81" t="str">
+      <c r="B71" t="str">
         <f>IF(D71&lt;&gt;"",VLOOKUP(D71,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A72" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B72" s="81" t="str">
+      <c r="A72" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B72" t="str">
         <f>IF(D72&lt;&gt;"",VLOOKUP(D72,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Strain and isolation information</v>
       </c>
-      <c r="C72" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D72" s="82" t="s">
+      <c r="C72" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>1113</v>
       </c>
-      <c r="E72" s="82"/>
-      <c r="F72" s="82" t="s">
+      <c r="E72" s="6"/>
+      <c r="F72" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G72" s="82"/>
-      <c r="H72" s="82" t="s">
+      <c r="G72" s="6"/>
+      <c r="H72" s="6" t="s">
         <v>1658</v>
       </c>
-      <c r="I72" s="82"/>
-      <c r="J72" s="82" t="s">
+      <c r="I72" s="6"/>
+      <c r="J72" s="6" t="s">
         <v>1107</v>
       </c>
-      <c r="K72" s="82" t="s">
+      <c r="K72" s="6" t="s">
         <v>1107</v>
       </c>
-      <c r="L72" s="82" t="s">
+      <c r="L72" s="6" t="s">
         <v>1113</v>
       </c>
-      <c r="M72" s="82" t="s">
+      <c r="M72" s="6" t="s">
         <v>1990</v>
       </c>
-      <c r="N72" s="82"/>
-      <c r="O72" s="82" t="s">
+      <c r="N72" s="6"/>
+      <c r="O72" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P72" s="82" t="s">
+      <c r="P72" s="6" t="s">
         <v>1656</v>
       </c>
-      <c r="Q72" s="82"/>
-      <c r="R72" s="82" t="s">
+      <c r="Q72" s="6"/>
+      <c r="R72" s="6" t="s">
         <v>1652</v>
       </c>
-      <c r="S72" s="83" t="s">
+      <c r="S72" s="5" t="s">
         <v>1659</v>
       </c>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="B73" s="81" t="str">
+      <c r="B73" t="str">
         <f>IF(D73&lt;&gt;"",VLOOKUP(D73,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v/>
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A74" s="82" t="b">
-        <v>1</v>
-      </c>
-      <c r="B74" s="81" t="str">
+      <c r="A74" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B74" t="str">
         <f>IF(D74&lt;&gt;"",VLOOKUP(D74,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Taxonomic identification information</v>
       </c>
-      <c r="C74" s="82" t="s">
-        <v>1809</v>
-      </c>
-      <c r="D74" s="82" t="s">
+      <c r="C74" s="6" t="s">
+        <v>1809</v>
+      </c>
+      <c r="D74" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E74" s="82"/>
-      <c r="F74" s="82" t="s">
+      <c r="E74" s="6"/>
+      <c r="F74" s="6" t="s">
         <v>1237</v>
       </c>
-      <c r="G74" s="82"/>
-      <c r="H74" s="82"/>
-      <c r="I74" s="82"/>
-      <c r="J74" s="82" t="s">
+      <c r="G74" s="6"/>
+      <c r="H74" s="6"/>
+      <c r="I74" s="6"/>
+      <c r="J74" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="K74" s="82" t="s">
+      <c r="K74" s="6" t="s">
         <v>1115</v>
       </c>
-      <c r="L74" s="82" t="s">
+      <c r="L74" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="M74" s="82" t="s">
+      <c r="M74" s="6" t="s">
         <v>2075</v>
       </c>
-      <c r="N74" s="82"/>
-      <c r="O74" s="82" t="s">
+      <c r="N74" s="6"/>
+      <c r="O74" s="6" t="s">
         <v>1037</v>
       </c>
-      <c r="P74" s="82" t="s">
+      <c r="P74" s="6" t="s">
         <v>1657</v>
       </c>
-      <c r="Q74" s="82"/>
-      <c r="R74" s="82" t="s">
+      <c r="Q74" s="6"/>
+      <c r="R74" s="6" t="s">
         <v>1655</v>
       </c>
-      <c r="S74" s="83" t="s">
+      <c r="S74" s="5" t="s">
         <v>1659</v>
       </c>
     </row>
@@ -37892,7 +37886,6 @@
       <c r="C28" t="s">
         <v>1809</v>
       </c>
-      <c r="D28" s="85"/>
       <c r="F28" t="s">
         <v>1400</v>
       </c>
@@ -37919,7 +37912,6 @@
       <c r="C29" t="s">
         <v>1809</v>
       </c>
-      <c r="D29" s="85"/>
       <c r="F29" t="s">
         <v>1400</v>
       </c>
@@ -37946,7 +37938,6 @@
       <c r="C30" t="s">
         <v>1809</v>
       </c>
-      <c r="D30" s="85"/>
       <c r="F30" t="s">
         <v>1400</v>
       </c>
@@ -37973,7 +37964,6 @@
       <c r="C31" t="s">
         <v>1809</v>
       </c>
-      <c r="D31" s="85"/>
       <c r="F31" t="s">
         <v>1400</v>
       </c>
@@ -63039,7 +63029,7 @@
         <v>1803</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>1791</v>
+        <v>2089</v>
       </c>
       <c r="M1" s="17" t="s">
         <v>1804</v>

</xml_diff>

<commit_message>
Removal of datasetID from organizations/instruments and contactID from instruments
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32979847-AEA8-4A44-B26C-105F0E4A8CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AD8CCF-E901-144F-917B-C6FBFA573CA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="160" yWindow="660" windowWidth="40800" windowHeight="20740" firstSheet="19" activeTab="22" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
   </bookViews>
@@ -39832,7 +39832,7 @@
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B30" t="str">
         <f>IF(D30&lt;&gt;"",VLOOKUP(D30,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
@@ -39862,7 +39862,7 @@
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B31" t="str">
         <f>IF(D31&lt;&gt;"",VLOOKUP(D31,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>

</xml_diff>

<commit_message>
Updates to PHA4GE to ODM mappings
</commit_message>
<xml_diff>
--- a/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
+++ b/odm_map_maker/data/mapping_config_files/pha4ge_to_odm_v2_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/odm_map_maker/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E194AF8-2581-3141-9B84-699B1BF5AD9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D6475E-DF38-194C-85F2-B12A319B9DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="40800" windowHeight="20740" firstSheet="10" activeTab="11" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="40800" windowHeight="20740" firstSheet="19" activeTab="28" xr2:uid="{D031FD9F-8EDE-1249-89E5-2C42697DC0B4}"/>
   </bookViews>
   <sheets>
     <sheet name="global_enums" sheetId="42" r:id="rId1"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9757" uniqueCount="2120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9776" uniqueCount="2122">
   <si>
     <t>Complete</t>
   </si>
@@ -6480,9 +6480,6 @@
     target = emap.collection_method</t>
   </si>
   <si>
-    <t>{ mirror_source: True }</t>
-  </si>
-  <si>
     <t>enumDerivationSettings</t>
   </si>
   <si>
@@ -6512,6 +6509,19 @@
   </si>
   <si>
     <t>{{quality control determination}}</t>
+  </si>
+  <si>
+    <t>{ mirror_source: False }</t>
+  </si>
+  <si>
+    <t>pooled</t>
+  </si>
+  <si>
+    <t>def is_pooled(values):
+    values = [v.lower().split('[')[0].strip() for v in values if isinstance(v, str)]
+    values = [v for v in values if v == "pooling specimens"]
+    return len(values) &gt; 0
+target = is_pooled(src.specimen_processing)</t>
   </si>
 </sst>
 </file>
@@ -6845,7 +6855,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -7002,6 +7012,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" customBuiltin="1"/>
@@ -21045,7 +21059,7 @@
         <v>6</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>2111</v>
+        <v>2110</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -21059,7 +21073,7 @@
         <v>441</v>
       </c>
       <c r="D2" t="s">
-        <v>2110</v>
+        <v>2119</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -26462,7 +26476,7 @@
         <v>1906</v>
       </c>
       <c r="S1" s="16" t="s">
-        <v>2118</v>
+        <v>2117</v>
       </c>
       <c r="T1" s="17" t="s">
         <v>1734</v>
@@ -32683,7 +32697,7 @@
         <v>2093</v>
       </c>
       <c r="S139" t="s">
-        <v>2119</v>
+        <v>2118</v>
       </c>
       <c r="T139" t="s">
         <v>1917</v>
@@ -35338,7 +35352,7 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E19831EB-F90F-BD49-AC5C-0138EB88F455}">
   <sheetPr codeName="Sheet14"/>
-  <dimension ref="A1:U74"/>
+  <dimension ref="A1:U75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
@@ -37372,54 +37386,59 @@
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A51" t="b">
+        <v>1</v>
+      </c>
       <c r="B51" t="str">
         <f>IF(D51&lt;&gt;"",VLOOKUP(D51,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Sample collection and processing</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D51" t="s">
+        <v>128</v>
+      </c>
+      <c r="E51" t="s">
+        <v>1127</v>
+      </c>
+      <c r="F51" t="s">
+        <v>1226</v>
+      </c>
+      <c r="J51" t="s">
+        <v>127</v>
+      </c>
+      <c r="K51" t="s">
+        <v>127</v>
+      </c>
+      <c r="L51" t="s">
+        <v>128</v>
+      </c>
+      <c r="M51" t="s">
+        <v>121</v>
+      </c>
+      <c r="N51" t="s">
+        <v>1506</v>
+      </c>
+      <c r="O51" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q51" s="8" t="s">
+        <v>2102</v>
+      </c>
+      <c r="R51" s="8"/>
+      <c r="S51" s="8"/>
+      <c r="T51" t="s">
+        <v>1513</v>
+      </c>
+      <c r="U51" t="s">
+        <v>1511</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A52" t="b">
-        <v>1</v>
-      </c>
       <c r="B52" t="str">
         <f>IF(D52&lt;&gt;"",VLOOKUP(D52,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>AMR detection information</v>
-      </c>
-      <c r="C52" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D52" t="s">
-        <v>1112</v>
-      </c>
-      <c r="F52" t="s">
-        <v>1226</v>
-      </c>
-      <c r="H52" t="s">
-        <v>1664</v>
-      </c>
-      <c r="J52" t="s">
-        <v>1105</v>
-      </c>
-      <c r="K52" t="s">
-        <v>1105</v>
-      </c>
-      <c r="L52" t="s">
-        <v>1112</v>
-      </c>
-      <c r="M52" t="s">
-        <v>2099</v>
-      </c>
-      <c r="O52" t="s">
-        <v>1027</v>
-      </c>
-      <c r="Q52" t="s">
-        <v>1528</v>
-      </c>
-      <c r="R52" t="s">
-        <v>1634</v>
-      </c>
-      <c r="T52" t="s">
-        <v>1529</v>
+        <v/>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.2">
@@ -37428,19 +37447,19 @@
       </c>
       <c r="B53" t="str">
         <f>IF(D53&lt;&gt;"",VLOOKUP(D53,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Bioinformatics and QC metrics</v>
+        <v>AMR detection information</v>
       </c>
       <c r="C53" t="s">
         <v>1751</v>
       </c>
       <c r="D53" t="s">
-        <v>13</v>
+        <v>1112</v>
       </c>
       <c r="F53" t="s">
         <v>1226</v>
       </c>
       <c r="H53" t="s">
-        <v>1661</v>
+        <v>1664</v>
       </c>
       <c r="J53" t="s">
         <v>1105</v>
@@ -37449,22 +37468,22 @@
         <v>1105</v>
       </c>
       <c r="L53" t="s">
-        <v>13</v>
+        <v>1112</v>
       </c>
       <c r="M53" t="s">
-        <v>121</v>
+        <v>2099</v>
       </c>
       <c r="O53" t="s">
         <v>1027</v>
       </c>
       <c r="Q53" t="s">
-        <v>1532</v>
+        <v>1528</v>
       </c>
       <c r="R53" t="s">
-        <v>1635</v>
+        <v>1634</v>
       </c>
       <c r="T53" t="s">
-        <v>1533</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.2">
@@ -37479,11 +37498,14 @@
         <v>1751</v>
       </c>
       <c r="D54" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F54" t="s">
         <v>1226</v>
       </c>
+      <c r="H54" t="s">
+        <v>1661</v>
+      </c>
       <c r="J54" t="s">
         <v>1105</v>
       </c>
@@ -37491,7 +37513,7 @@
         <v>1105</v>
       </c>
       <c r="L54" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M54" t="s">
         <v>121</v>
@@ -37500,10 +37522,10 @@
         <v>1027</v>
       </c>
       <c r="Q54" t="s">
-        <v>1534</v>
+        <v>1532</v>
       </c>
       <c r="R54" t="s">
-        <v>1636</v>
+        <v>1635</v>
       </c>
       <c r="T54" t="s">
         <v>1533</v>
@@ -37521,7 +37543,7 @@
         <v>1751</v>
       </c>
       <c r="D55" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F55" t="s">
         <v>1226</v>
@@ -37533,7 +37555,7 @@
         <v>1105</v>
       </c>
       <c r="L55" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="M55" t="s">
         <v>121</v>
@@ -37542,10 +37564,10 @@
         <v>1027</v>
       </c>
       <c r="Q55" t="s">
-        <v>1535</v>
+        <v>1534</v>
       </c>
       <c r="R55" t="s">
-        <v>1637</v>
+        <v>1636</v>
       </c>
       <c r="T55" t="s">
         <v>1533</v>
@@ -37563,7 +37585,7 @@
         <v>1751</v>
       </c>
       <c r="D56" t="s">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="F56" t="s">
         <v>1226</v>
@@ -37575,7 +37597,7 @@
         <v>1105</v>
       </c>
       <c r="L56" t="s">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="M56" t="s">
         <v>121</v>
@@ -37584,10 +37606,10 @@
         <v>1027</v>
       </c>
       <c r="Q56" t="s">
-        <v>1539</v>
+        <v>1535</v>
       </c>
       <c r="R56" t="s">
-        <v>1638</v>
+        <v>1637</v>
       </c>
       <c r="T56" t="s">
         <v>1533</v>
@@ -37605,14 +37627,11 @@
         <v>1751</v>
       </c>
       <c r="D57" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F57" t="s">
         <v>1226</v>
       </c>
-      <c r="H57" t="s">
-        <v>1662</v>
-      </c>
       <c r="J57" t="s">
         <v>1105</v>
       </c>
@@ -37620,7 +37639,7 @@
         <v>1105</v>
       </c>
       <c r="L57" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="M57" t="s">
         <v>121</v>
@@ -37629,10 +37648,10 @@
         <v>1027</v>
       </c>
       <c r="Q57" t="s">
-        <v>1540</v>
+        <v>1539</v>
       </c>
       <c r="R57" t="s">
-        <v>1639</v>
+        <v>1638</v>
       </c>
       <c r="T57" t="s">
         <v>1533</v>
@@ -37644,19 +37663,19 @@
       </c>
       <c r="B58" t="str">
         <f>IF(D58&lt;&gt;"",VLOOKUP(D58,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Lineage/clade information</v>
+        <v>Bioinformatics and QC metrics</v>
       </c>
       <c r="C58" t="s">
         <v>1751</v>
       </c>
       <c r="D58" t="s">
-        <v>1119</v>
+        <v>95</v>
       </c>
       <c r="F58" t="s">
         <v>1226</v>
       </c>
       <c r="H58" t="s">
-        <v>2021</v>
+        <v>1662</v>
       </c>
       <c r="J58" t="s">
         <v>1105</v>
@@ -37665,7 +37684,7 @@
         <v>1105</v>
       </c>
       <c r="L58" t="s">
-        <v>1119</v>
+        <v>95</v>
       </c>
       <c r="M58" t="s">
         <v>121</v>
@@ -37674,224 +37693,218 @@
         <v>1027</v>
       </c>
       <c r="Q58" t="s">
-        <v>1541</v>
+        <v>1540</v>
       </c>
       <c r="R58" t="s">
-        <v>1640</v>
+        <v>1639</v>
       </c>
       <c r="T58" t="s">
-        <v>1542</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A59" t="b">
+        <v>1</v>
+      </c>
       <c r="B59" t="str">
         <f>IF(D59&lt;&gt;"",VLOOKUP(D59,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Lineage/clade information</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1119</v>
+      </c>
+      <c r="F59" t="s">
+        <v>1226</v>
+      </c>
+      <c r="H59" t="s">
+        <v>2021</v>
+      </c>
+      <c r="J59" t="s">
+        <v>1105</v>
+      </c>
+      <c r="K59" t="s">
+        <v>1105</v>
+      </c>
+      <c r="L59" t="s">
+        <v>1119</v>
+      </c>
+      <c r="M59" t="s">
+        <v>121</v>
+      </c>
+      <c r="O59" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>1541</v>
+      </c>
+      <c r="R59" t="s">
+        <v>1640</v>
+      </c>
+      <c r="T59" t="s">
+        <v>1542</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A60" t="b">
-        <v>1</v>
-      </c>
       <c r="B60" t="str">
         <f>IF(D60&lt;&gt;"",VLOOKUP(D60,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Sample collection and processing</v>
-      </c>
-      <c r="C60" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D60" t="s">
-        <v>1784</v>
-      </c>
-      <c r="F60" t="s">
-        <v>1226</v>
-      </c>
-      <c r="H60" t="s">
-        <v>1951</v>
-      </c>
-      <c r="J60" t="s">
-        <v>127</v>
-      </c>
-      <c r="K60" t="s">
-        <v>127</v>
-      </c>
-      <c r="L60" t="s">
-        <v>1784</v>
-      </c>
-      <c r="M60" t="s">
-        <v>121</v>
-      </c>
-      <c r="O60" t="s">
-        <v>1027</v>
-      </c>
-      <c r="Q60" t="s">
-        <v>1549</v>
-      </c>
-      <c r="R60" t="s">
-        <v>1952</v>
-      </c>
-      <c r="T60" t="s">
-        <v>1550</v>
+        <v/>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A61" t="b">
+        <v>1</v>
+      </c>
       <c r="B61" t="str">
         <f>IF(D61&lt;&gt;"",VLOOKUP(D61,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Sample collection and processing</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1784</v>
+      </c>
+      <c r="F61" t="s">
+        <v>1226</v>
+      </c>
+      <c r="H61" t="s">
+        <v>1951</v>
+      </c>
+      <c r="J61" t="s">
+        <v>127</v>
+      </c>
+      <c r="K61" t="s">
+        <v>127</v>
+      </c>
+      <c r="L61" t="s">
+        <v>1784</v>
+      </c>
+      <c r="M61" t="s">
+        <v>121</v>
+      </c>
+      <c r="O61" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>1549</v>
+      </c>
+      <c r="R61" t="s">
+        <v>1952</v>
+      </c>
+      <c r="T61" t="s">
+        <v>1550</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A62" t="b">
-        <v>1</v>
-      </c>
       <c r="B62" t="str">
         <f>IF(D62&lt;&gt;"",VLOOKUP(D62,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Sample collection and processing</v>
-      </c>
-      <c r="C62" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D62" t="s">
-        <v>125</v>
-      </c>
-      <c r="F62" t="s">
-        <v>1226</v>
-      </c>
-      <c r="G62" s="9"/>
-      <c r="H62" t="s">
-        <v>1681</v>
-      </c>
-      <c r="J62" t="s">
-        <v>127</v>
-      </c>
-      <c r="K62" t="s">
-        <v>127</v>
-      </c>
-      <c r="L62" t="s">
-        <v>125</v>
-      </c>
-      <c r="M62" t="s">
-        <v>121</v>
-      </c>
-      <c r="O62" t="s">
-        <v>1027</v>
-      </c>
-      <c r="Q62" t="s">
-        <v>1560</v>
-      </c>
-      <c r="R62" t="s">
-        <v>1559</v>
-      </c>
-      <c r="T62" t="s">
-        <v>1561</v>
+        <v/>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A63" t="b">
+        <v>1</v>
+      </c>
       <c r="B63" t="str">
         <f>IF(D63&lt;&gt;"",VLOOKUP(D63,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Sample collection and processing</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D63" t="s">
+        <v>125</v>
+      </c>
+      <c r="F63" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G63" s="9"/>
+      <c r="H63" t="s">
+        <v>1681</v>
+      </c>
+      <c r="J63" t="s">
+        <v>127</v>
+      </c>
+      <c r="K63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L63" t="s">
+        <v>125</v>
+      </c>
+      <c r="M63" t="s">
+        <v>121</v>
+      </c>
+      <c r="O63" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>1560</v>
+      </c>
+      <c r="R63" t="s">
+        <v>1559</v>
+      </c>
+      <c r="T63" t="s">
+        <v>1561</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A64" t="b">
-        <v>1</v>
-      </c>
       <c r="B64" t="str">
         <f>IF(D64&lt;&gt;"",VLOOKUP(D64,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Sequence information</v>
-      </c>
-      <c r="C64" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D64" t="s">
-        <v>89</v>
-      </c>
-      <c r="F64" t="s">
-        <v>1226</v>
-      </c>
-      <c r="H64" t="s">
-        <v>1684</v>
-      </c>
-      <c r="J64" t="s">
-        <v>1105</v>
-      </c>
-      <c r="K64" t="s">
-        <v>1105</v>
-      </c>
-      <c r="L64" t="s">
-        <v>89</v>
-      </c>
-      <c r="M64" t="s">
-        <v>121</v>
-      </c>
-      <c r="O64" t="s">
-        <v>1027</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>1573</v>
-      </c>
-      <c r="R64" t="s">
-        <v>1572</v>
-      </c>
-      <c r="T64" t="s">
-        <v>1574</v>
+        <v/>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A65" t="b">
+        <v>1</v>
+      </c>
       <c r="B65" t="str">
         <f>IF(D65&lt;&gt;"",VLOOKUP(D65,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Sequence information</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D65" t="s">
+        <v>89</v>
+      </c>
+      <c r="F65" t="s">
+        <v>1226</v>
+      </c>
+      <c r="H65" t="s">
+        <v>1684</v>
+      </c>
+      <c r="J65" t="s">
+        <v>1105</v>
+      </c>
+      <c r="K65" t="s">
+        <v>1105</v>
+      </c>
+      <c r="L65" t="s">
+        <v>89</v>
+      </c>
+      <c r="M65" t="s">
+        <v>121</v>
+      </c>
+      <c r="O65" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>1573</v>
+      </c>
+      <c r="R65" t="s">
+        <v>1572</v>
+      </c>
+      <c r="T65" t="s">
+        <v>1574</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A66" t="b">
-        <v>1</v>
-      </c>
       <c r="B66" t="str">
         <f>IF(D66&lt;&gt;"",VLOOKUP(D66,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Sequence information</v>
-      </c>
-      <c r="C66" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D66" t="s">
-        <v>1107</v>
-      </c>
-      <c r="E66" t="s">
-        <v>1937</v>
-      </c>
-      <c r="F66" t="s">
-        <v>1226</v>
-      </c>
-      <c r="G66" t="s">
-        <v>1578</v>
-      </c>
-      <c r="I66" t="s">
-        <v>19</v>
-      </c>
-      <c r="J66" t="s">
-        <v>1105</v>
-      </c>
-      <c r="K66" t="s">
-        <v>1105</v>
-      </c>
-      <c r="L66" t="s">
-        <v>1107</v>
-      </c>
-      <c r="M66" t="s">
-        <v>121</v>
-      </c>
-      <c r="O66" t="s">
-        <v>1027</v>
-      </c>
-      <c r="Q66" t="s">
-        <v>1576</v>
-      </c>
-      <c r="R66" t="s">
-        <v>1660</v>
-      </c>
-      <c r="T66" t="s">
-        <v>1583</v>
+        <v/>
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.2">
@@ -37909,13 +37922,13 @@
         <v>1107</v>
       </c>
       <c r="E67" t="s">
-        <v>1577</v>
+        <v>1937</v>
       </c>
       <c r="F67" t="s">
         <v>1226</v>
       </c>
       <c r="G67" t="s">
-        <v>1580</v>
+        <v>1578</v>
       </c>
       <c r="I67" t="s">
         <v>19</v>
@@ -37960,13 +37973,13 @@
         <v>1107</v>
       </c>
       <c r="E68" t="s">
-        <v>1936</v>
+        <v>1577</v>
       </c>
       <c r="F68" t="s">
         <v>1226</v>
       </c>
       <c r="G68" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="I68" t="s">
         <v>19</v>
@@ -38011,13 +38024,13 @@
         <v>1107</v>
       </c>
       <c r="E69" t="s">
-        <v>1934</v>
+        <v>1936</v>
       </c>
       <c r="F69" t="s">
         <v>1226</v>
       </c>
       <c r="G69" t="s">
-        <v>1581</v>
+        <v>1579</v>
       </c>
       <c r="I69" t="s">
         <v>19</v>
@@ -38062,13 +38075,13 @@
         <v>1107</v>
       </c>
       <c r="E70" t="s">
-        <v>1935</v>
+        <v>1934</v>
       </c>
       <c r="F70" t="s">
         <v>1226</v>
       </c>
       <c r="G70" t="s">
-        <v>1582</v>
+        <v>1581</v>
       </c>
       <c r="I70" t="s">
         <v>19</v>
@@ -38099,101 +38112,152 @@
       </c>
     </row>
     <row r="71" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A71" t="b">
+        <v>1</v>
+      </c>
       <c r="B71" t="str">
         <f>IF(D71&lt;&gt;"",VLOOKUP(D71,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Sequence information</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D71" t="s">
+        <v>1107</v>
+      </c>
+      <c r="E71" t="s">
+        <v>1935</v>
+      </c>
+      <c r="F71" t="s">
+        <v>1226</v>
+      </c>
+      <c r="G71" t="s">
+        <v>1582</v>
+      </c>
+      <c r="I71" t="s">
+        <v>19</v>
+      </c>
+      <c r="J71" t="s">
+        <v>1105</v>
+      </c>
+      <c r="K71" t="s">
+        <v>1105</v>
+      </c>
+      <c r="L71" t="s">
+        <v>1107</v>
+      </c>
+      <c r="M71" t="s">
+        <v>121</v>
+      </c>
+      <c r="O71" t="s">
+        <v>1027</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>1576</v>
+      </c>
+      <c r="R71" t="s">
+        <v>1660</v>
+      </c>
+      <c r="T71" t="s">
+        <v>1583</v>
       </c>
     </row>
     <row r="72" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A72" t="b">
-        <v>1</v>
-      </c>
       <c r="B72" t="str">
         <f>IF(D72&lt;&gt;"",VLOOKUP(D72,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v>Strain and isolation information</v>
-      </c>
-      <c r="C72" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D72" t="s">
-        <v>1103</v>
-      </c>
-      <c r="F72" t="s">
-        <v>1226</v>
-      </c>
-      <c r="J72" t="s">
-        <v>1097</v>
-      </c>
-      <c r="K72" t="s">
-        <v>1097</v>
-      </c>
-      <c r="L72" t="s">
-        <v>1103</v>
-      </c>
-      <c r="M72" t="s">
-        <v>2101</v>
-      </c>
-      <c r="O72" t="s">
-        <v>1027</v>
-      </c>
-      <c r="P72" t="s">
-        <v>1609</v>
-      </c>
-      <c r="R72" t="s">
-        <v>1605</v>
-      </c>
-      <c r="T72" t="s">
-        <v>1611</v>
+        <v/>
       </c>
     </row>
     <row r="73" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A73" t="b">
+        <v>1</v>
+      </c>
       <c r="B73" t="str">
         <f>IF(D73&lt;&gt;"",VLOOKUP(D73,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
-        <v/>
+        <v>Strain and isolation information</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D73" t="s">
+        <v>1103</v>
+      </c>
+      <c r="F73" t="s">
+        <v>1226</v>
+      </c>
+      <c r="J73" t="s">
+        <v>1097</v>
+      </c>
+      <c r="K73" t="s">
+        <v>1097</v>
+      </c>
+      <c r="L73" t="s">
+        <v>1103</v>
+      </c>
+      <c r="M73" t="s">
+        <v>2101</v>
+      </c>
+      <c r="O73" t="s">
+        <v>1027</v>
+      </c>
+      <c r="P73" t="s">
+        <v>1609</v>
+      </c>
+      <c r="R73" t="s">
+        <v>1605</v>
+      </c>
+      <c r="T73" t="s">
+        <v>1611</v>
       </c>
     </row>
     <row r="74" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A74" t="b">
-        <v>1</v>
-      </c>
       <c r="B74" t="str">
         <f>IF(D74&lt;&gt;"",VLOOKUP(D74,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A75" t="b">
+        <v>1</v>
+      </c>
+      <c r="B75" t="str">
+        <f>IF(D75&lt;&gt;"",VLOOKUP(D75,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
         <v>Taxonomic identification information</v>
       </c>
-      <c r="C74" t="s">
-        <v>1751</v>
-      </c>
-      <c r="D74" t="s">
+      <c r="C75" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D75" t="s">
         <v>91</v>
       </c>
-      <c r="F74" t="s">
+      <c r="F75" t="s">
         <v>1226</v>
       </c>
-      <c r="H74" t="s">
+      <c r="H75" t="s">
         <v>2023</v>
       </c>
-      <c r="J74" t="s">
+      <c r="J75" t="s">
         <v>1105</v>
       </c>
-      <c r="K74" t="s">
+      <c r="K75" t="s">
         <v>1105</v>
       </c>
-      <c r="L74" t="s">
+      <c r="L75" t="s">
         <v>91</v>
       </c>
-      <c r="M74" t="s">
+      <c r="M75" t="s">
         <v>121</v>
       </c>
-      <c r="O74" t="s">
+      <c r="O75" t="s">
         <v>1027</v>
       </c>
-      <c r="P74" t="s">
+      <c r="P75" t="s">
         <v>1610</v>
       </c>
-      <c r="R74" t="s">
+      <c r="R75" t="s">
         <v>1608</v>
       </c>
-      <c r="T74" t="s">
+      <c r="T75" t="s">
         <v>1611</v>
       </c>
     </row>
@@ -40390,7 +40454,7 @@
         <v>1250</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>2117</v>
+        <v>2116</v>
       </c>
       <c r="M17" s="15" t="s">
         <v>2095</v>
@@ -42701,7 +42765,7 @@
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E39206-1F1B-2D4B-82A5-94676E67F7A4}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
@@ -43478,6 +43542,36 @@
       </c>
       <c r="P20" s="24" t="s">
         <v>1754</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" s="78" customFormat="1" ht="119" x14ac:dyDescent="0.2">
+      <c r="B22" s="78" t="b">
+        <v>1</v>
+      </c>
+      <c r="C22" s="78" t="b">
+        <v>1</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="78" t="str">
+        <f>IF(G22&lt;&gt;"",VLOOKUP(G22,PHA4GEVars!$A$7:$B$241,2,FALSE),"")</f>
+        <v>Sample collection and processing</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>1751</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>1178</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>2120</v>
+      </c>
+      <c r="L22" s="79" t="s">
+        <v>2121</v>
       </c>
     </row>
   </sheetData>
@@ -54585,7 +54679,7 @@
         <v>1178</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>2114</v>
+        <v>2113</v>
       </c>
       <c r="H3" s="28" t="s">
         <v>127</v>
@@ -64381,10 +64475,10 @@
         <v>1957</v>
       </c>
       <c r="J1" s="10" t="s">
+        <v>2114</v>
+      </c>
+      <c r="K1" s="10" t="s">
         <v>2115</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>2116</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>1964</v>
@@ -64643,7 +64737,7 @@
       </c>
       <c r="L4" s="15"/>
       <c r="M4" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N4" s="15"/>
       <c r="O4" s="18" t="s">
@@ -64685,7 +64779,7 @@
       </c>
       <c r="L5" s="15"/>
       <c r="M5" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N5" s="15"/>
       <c r="O5" s="18" t="s">
@@ -64727,7 +64821,7 @@
       </c>
       <c r="L6" s="15"/>
       <c r="M6" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N6" s="15"/>
       <c r="O6" s="18" t="s">
@@ -64769,7 +64863,7 @@
       </c>
       <c r="L7" s="15"/>
       <c r="M7" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N7" s="15"/>
       <c r="O7" s="18" t="s">
@@ -64811,7 +64905,7 @@
       </c>
       <c r="L8" s="15"/>
       <c r="M8" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N8" s="15"/>
       <c r="O8" s="18" t="s">
@@ -64853,7 +64947,7 @@
       </c>
       <c r="L9" s="15"/>
       <c r="M9" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N9" s="15"/>
       <c r="O9" s="18" t="s">
@@ -64895,7 +64989,7 @@
       </c>
       <c r="L10" s="15"/>
       <c r="M10" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N10" s="15"/>
       <c r="O10" s="18" t="s">
@@ -64937,7 +65031,7 @@
       </c>
       <c r="L11" s="15"/>
       <c r="M11" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N11" s="15"/>
       <c r="O11" s="18" t="s">
@@ -64979,7 +65073,7 @@
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N12" s="15"/>
       <c r="O12" s="18" t="s">
@@ -65021,7 +65115,7 @@
       </c>
       <c r="L13" s="15"/>
       <c r="M13" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N13" s="15"/>
       <c r="O13" s="18" t="s">
@@ -65063,7 +65157,7 @@
       </c>
       <c r="L14" s="15"/>
       <c r="M14" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N14" s="15"/>
       <c r="O14" s="18" t="s">
@@ -65105,7 +65199,7 @@
       </c>
       <c r="L15" s="15"/>
       <c r="M15" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N15" s="15"/>
       <c r="O15" s="18" t="s">
@@ -65147,7 +65241,7 @@
       </c>
       <c r="L16" s="15"/>
       <c r="M16" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="18" t="s">
@@ -65189,7 +65283,7 @@
       </c>
       <c r="L17" s="15"/>
       <c r="M17" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N17" s="15"/>
       <c r="O17" s="18" t="s">
@@ -65231,7 +65325,7 @@
       </c>
       <c r="L18" s="15"/>
       <c r="M18" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N18" s="15"/>
       <c r="O18" s="18" t="s">
@@ -65273,7 +65367,7 @@
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N19" s="15"/>
       <c r="O19" s="18" t="s">
@@ -65315,7 +65409,7 @@
       </c>
       <c r="L20" s="15"/>
       <c r="M20" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N20" s="15"/>
       <c r="O20" s="18" t="s">
@@ -65357,7 +65451,7 @@
       </c>
       <c r="L21" s="15"/>
       <c r="M21" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N21" s="15"/>
       <c r="O21" s="18" t="s">
@@ -65399,7 +65493,7 @@
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N22" s="15"/>
       <c r="O22" s="18" t="s">
@@ -65441,7 +65535,7 @@
       </c>
       <c r="L23" s="15"/>
       <c r="M23" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N23" s="15"/>
       <c r="O23" s="18" t="s">
@@ -65483,7 +65577,7 @@
       </c>
       <c r="L24" s="15"/>
       <c r="M24" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N24" s="15"/>
       <c r="O24" s="18" t="s">
@@ -65525,7 +65619,7 @@
       </c>
       <c r="L25" s="15"/>
       <c r="M25" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N25" s="15"/>
       <c r="O25" s="18" t="s">
@@ -65567,7 +65661,7 @@
       </c>
       <c r="L26" s="15"/>
       <c r="M26" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N26" s="15"/>
       <c r="O26" s="18" t="s">
@@ -65609,7 +65703,7 @@
       </c>
       <c r="L27" s="15"/>
       <c r="M27" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N27" s="15"/>
       <c r="O27" s="18" t="s">
@@ -65651,7 +65745,7 @@
       </c>
       <c r="L28" s="15"/>
       <c r="M28" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N28" s="15"/>
       <c r="O28" s="18" t="s">
@@ -65693,7 +65787,7 @@
       </c>
       <c r="L29" s="15"/>
       <c r="M29" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N29" s="15"/>
       <c r="O29" s="18" t="s">
@@ -65735,7 +65829,7 @@
       </c>
       <c r="L30" s="15"/>
       <c r="M30" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N30" s="15"/>
       <c r="O30" s="18" t="s">
@@ -65777,7 +65871,7 @@
       </c>
       <c r="L31" s="15"/>
       <c r="M31" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N31" s="15"/>
       <c r="O31" s="18" t="s">
@@ -65819,7 +65913,7 @@
       </c>
       <c r="L32" s="15"/>
       <c r="M32" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N32" s="15"/>
       <c r="O32" s="18" t="s">
@@ -65861,7 +65955,7 @@
       </c>
       <c r="L33" s="15"/>
       <c r="M33" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N33" s="15"/>
       <c r="O33" s="18" t="s">
@@ -65903,7 +65997,7 @@
       </c>
       <c r="L34" s="15"/>
       <c r="M34" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N34" s="15"/>
       <c r="O34" s="18" t="s">
@@ -65945,7 +66039,7 @@
       </c>
       <c r="L35" s="15"/>
       <c r="M35" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N35" s="15"/>
       <c r="O35" s="18" t="s">
@@ -65987,7 +66081,7 @@
       </c>
       <c r="L36" s="15"/>
       <c r="M36" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N36" s="15"/>
       <c r="O36" s="18" t="s">
@@ -66029,7 +66123,7 @@
       </c>
       <c r="L37" s="15"/>
       <c r="M37" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N37" s="15"/>
       <c r="O37" s="18" t="s">
@@ -66071,7 +66165,7 @@
       </c>
       <c r="L38" s="15"/>
       <c r="M38" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N38" s="15"/>
       <c r="O38" s="18" t="s">
@@ -66113,7 +66207,7 @@
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N39" s="15"/>
       <c r="O39" s="18" t="s">
@@ -66155,7 +66249,7 @@
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N40" s="15"/>
       <c r="O40" s="18" t="s">
@@ -66197,7 +66291,7 @@
       </c>
       <c r="L41" s="15"/>
       <c r="M41" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N41" s="15"/>
       <c r="O41" s="18" t="s">
@@ -66239,7 +66333,7 @@
       </c>
       <c r="L42" s="15"/>
       <c r="M42" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N42" s="15"/>
       <c r="O42" s="18" t="s">
@@ -66281,7 +66375,7 @@
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N43" s="15"/>
       <c r="O43" s="18" t="s">
@@ -66323,7 +66417,7 @@
       </c>
       <c r="L44" s="15"/>
       <c r="M44" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N44" s="15"/>
       <c r="O44" s="18" t="s">
@@ -66365,7 +66459,7 @@
       </c>
       <c r="L45" s="15"/>
       <c r="M45" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N45" s="15"/>
       <c r="O45" s="18" t="s">
@@ -66407,7 +66501,7 @@
       </c>
       <c r="L46" s="15"/>
       <c r="M46" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N46" s="15"/>
       <c r="O46" s="18" t="s">
@@ -66449,7 +66543,7 @@
       </c>
       <c r="L47" s="15"/>
       <c r="M47" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N47" s="15"/>
       <c r="O47" s="18" t="s">
@@ -66491,7 +66585,7 @@
       </c>
       <c r="L48" s="15"/>
       <c r="M48" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N48" s="15"/>
       <c r="O48" s="18" t="s">
@@ -66533,7 +66627,7 @@
       </c>
       <c r="L49" s="15"/>
       <c r="M49" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N49" s="15"/>
       <c r="O49" s="18" t="s">
@@ -66575,7 +66669,7 @@
       </c>
       <c r="L50" s="15"/>
       <c r="M50" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N50" s="15"/>
       <c r="O50" s="18" t="s">
@@ -66617,7 +66711,7 @@
       </c>
       <c r="L51" s="15"/>
       <c r="M51" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N51" s="15"/>
       <c r="O51" s="18" t="s">
@@ -66659,7 +66753,7 @@
       </c>
       <c r="L52" s="15"/>
       <c r="M52" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N52" s="15"/>
       <c r="O52" s="18" t="s">
@@ -66701,7 +66795,7 @@
       </c>
       <c r="L53" s="15"/>
       <c r="M53" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N53" s="15"/>
       <c r="O53" s="18" t="s">
@@ -66743,7 +66837,7 @@
       </c>
       <c r="L54" s="15"/>
       <c r="M54" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N54" s="15"/>
       <c r="O54" s="18" t="s">
@@ -66785,7 +66879,7 @@
       </c>
       <c r="L55" s="15"/>
       <c r="M55" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N55" s="15"/>
       <c r="O55" s="18" t="s">
@@ -66827,7 +66921,7 @@
       </c>
       <c r="L56" s="15"/>
       <c r="M56" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N56" s="15"/>
       <c r="O56" s="18" t="s">
@@ -66869,7 +66963,7 @@
       </c>
       <c r="L57" s="15"/>
       <c r="M57" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N57" s="15"/>
       <c r="O57" s="18" t="s">
@@ -66911,7 +67005,7 @@
       </c>
       <c r="L58" s="15"/>
       <c r="M58" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N58" s="15"/>
       <c r="O58" s="18" t="s">
@@ -66953,7 +67047,7 @@
       </c>
       <c r="L59" s="15"/>
       <c r="M59" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N59" s="15"/>
       <c r="O59" s="18" t="s">
@@ -66995,7 +67089,7 @@
       </c>
       <c r="L60" s="15"/>
       <c r="M60" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N60" s="15"/>
       <c r="O60" s="18" t="s">
@@ -67037,7 +67131,7 @@
       </c>
       <c r="L61" s="15"/>
       <c r="M61" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N61" s="15"/>
       <c r="O61" s="18" t="s">
@@ -67079,7 +67173,7 @@
       </c>
       <c r="L62" s="15"/>
       <c r="M62" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N62" s="15"/>
       <c r="O62" s="18" t="s">
@@ -67121,7 +67215,7 @@
       </c>
       <c r="L63" s="15"/>
       <c r="M63" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N63" s="15"/>
       <c r="O63" s="18" t="s">
@@ -67163,7 +67257,7 @@
       </c>
       <c r="L64" s="15"/>
       <c r="M64" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N64" s="15"/>
       <c r="O64" s="18" t="s">
@@ -67205,7 +67299,7 @@
       </c>
       <c r="L65" s="15"/>
       <c r="M65" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N65" s="15"/>
       <c r="O65" s="18" t="s">
@@ -67247,7 +67341,7 @@
       </c>
       <c r="L66" s="15"/>
       <c r="M66" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N66" s="15"/>
       <c r="O66" s="18" t="s">
@@ -67289,7 +67383,7 @@
       </c>
       <c r="L67" s="15"/>
       <c r="M67" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N67" s="15"/>
       <c r="O67" s="18" t="s">
@@ -67331,7 +67425,7 @@
       </c>
       <c r="L68" s="15"/>
       <c r="M68" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N68" s="15"/>
       <c r="O68" s="18" t="s">
@@ -67373,7 +67467,7 @@
       </c>
       <c r="L69" s="15"/>
       <c r="M69" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N69" s="15"/>
       <c r="O69" s="18" t="s">
@@ -67415,7 +67509,7 @@
       </c>
       <c r="L70" s="15"/>
       <c r="M70" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N70" s="15"/>
       <c r="O70" s="18" t="s">
@@ -67457,7 +67551,7 @@
       </c>
       <c r="L71" s="15"/>
       <c r="M71" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N71" s="15"/>
       <c r="O71" s="18" t="s">
@@ -67499,7 +67593,7 @@
       </c>
       <c r="L72" s="15"/>
       <c r="M72" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N72" s="15"/>
       <c r="O72" s="18" t="s">
@@ -67541,7 +67635,7 @@
       </c>
       <c r="L73" s="15"/>
       <c r="M73" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N73" s="15"/>
       <c r="O73" s="18" t="s">
@@ -67583,7 +67677,7 @@
       </c>
       <c r="L74" s="15"/>
       <c r="M74" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N74" s="15"/>
       <c r="O74" s="18" t="s">
@@ -67625,7 +67719,7 @@
       </c>
       <c r="L75" s="15"/>
       <c r="M75" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N75" s="15"/>
       <c r="O75" s="18" t="s">
@@ -67667,7 +67761,7 @@
       </c>
       <c r="L76" s="15"/>
       <c r="M76" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N76" s="15"/>
       <c r="O76" s="18" t="s">
@@ -67709,7 +67803,7 @@
       </c>
       <c r="L77" s="15"/>
       <c r="M77" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N77" s="15"/>
       <c r="O77" s="18" t="s">
@@ -67751,7 +67845,7 @@
       </c>
       <c r="L78" s="15"/>
       <c r="M78" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N78" s="15"/>
       <c r="O78" s="18" t="s">
@@ -67793,7 +67887,7 @@
       </c>
       <c r="L79" s="15"/>
       <c r="M79" s="15" t="s">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="N79" s="15"/>
       <c r="O79" s="18" t="s">
@@ -67855,7 +67949,7 @@
       </c>
       <c r="L81" s="15"/>
       <c r="M81" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N81" s="15"/>
       <c r="O81" s="18" t="s">
@@ -67897,7 +67991,7 @@
       </c>
       <c r="L82" s="15"/>
       <c r="M82" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N82" s="15"/>
       <c r="O82" s="18" t="s">
@@ -67939,7 +68033,7 @@
       </c>
       <c r="L83" s="15"/>
       <c r="M83" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N83" s="15"/>
       <c r="O83" s="18" t="s">
@@ -67981,7 +68075,7 @@
       </c>
       <c r="L84" s="15"/>
       <c r="M84" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N84" s="15"/>
       <c r="O84" s="18" t="s">
@@ -68023,7 +68117,7 @@
       </c>
       <c r="L85" s="15"/>
       <c r="M85" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N85" s="15"/>
       <c r="O85" s="18" t="s">
@@ -68065,7 +68159,7 @@
       </c>
       <c r="L86" s="15"/>
       <c r="M86" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N86" s="15"/>
       <c r="O86" s="18" t="s">
@@ -68107,7 +68201,7 @@
       </c>
       <c r="L87" s="15"/>
       <c r="M87" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N87" s="15"/>
       <c r="O87" s="18" t="s">
@@ -68149,7 +68243,7 @@
       </c>
       <c r="L88" s="15"/>
       <c r="M88" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N88" s="15"/>
       <c r="O88" s="18" t="s">
@@ -68191,7 +68285,7 @@
       </c>
       <c r="L89" s="15"/>
       <c r="M89" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N89" s="15"/>
       <c r="O89" s="18" t="s">
@@ -68233,7 +68327,7 @@
       </c>
       <c r="L90" s="15"/>
       <c r="M90" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N90" s="15"/>
       <c r="O90" s="18" t="s">
@@ -68275,7 +68369,7 @@
       </c>
       <c r="L91" s="15"/>
       <c r="M91" s="15" t="s">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="N91" s="15"/>
       <c r="O91" s="18" t="s">

</xml_diff>